<commit_message>
Save Movement Data into CSV
</commit_message>
<xml_diff>
--- a/25_26_Jahresplanung_Schule.xlsx
+++ b/25_26_Jahresplanung_Schule.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/05fd09ff656560cc/Dokumente/Diplomprojekt/FormerGlove/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\daned\OneDrive\Dokumente\Diplomprojekt\FormerGlove\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="104" documentId="8_{78F0A12D-8FAF-4DAF-A002-1C4848C1BD15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50266EF2-83AA-4670-8287-1EEBE8F68C2F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4309F77D-7632-4CB7-BF33-0B440E7BF5F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{48A84E54-BAB7-6C4B-B78A-044ECBD93EA1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
   <si>
     <t>KW</t>
   </si>
@@ -145,6 +145,24 @@
   </si>
   <si>
     <t>3D-Modell, µC-App Schnittstelle, Code für Datenübertragung zu Edge Impulse</t>
+  </si>
+  <si>
+    <t>Edge Impulse, App-Development</t>
+  </si>
+  <si>
+    <t>Meilenstein erreicht: µC kommunizieren miteinander und können Daten an App senden, App gibt erhaltene Werte aus</t>
+  </si>
+  <si>
+    <t>Nicla Sense ME + Akku mit Gehäusen an den Handschuhen montiert</t>
+  </si>
+  <si>
+    <t>Jugend innovativ Einreichung, App programmiert</t>
+  </si>
+  <si>
+    <t>Zeitungsartikel, Plakat, Batteriecode, App programmiert</t>
+  </si>
+  <si>
+    <t>Batteriecode, App programmiert</t>
   </si>
 </sst>
 </file>
@@ -330,9 +348,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -341,6 +356,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -361,6 +379,15 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
@@ -368,15 +395,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -393,10 +411,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -736,7 +750,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="28" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="8"/>
@@ -744,7 +758,7 @@
       <c r="D2" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="22" t="s">
+      <c r="E2" s="25" t="s">
         <v>22</v>
       </c>
       <c r="F2" s="21">
@@ -764,11 +778,11 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="25"/>
+      <c r="A3" s="28"/>
       <c r="B3" s="8"/>
       <c r="C3" s="2"/>
       <c r="D3" s="23"/>
-      <c r="E3" s="23"/>
+      <c r="E3" s="26"/>
       <c r="F3" s="21"/>
       <c r="G3" s="30"/>
       <c r="H3" s="21"/>
@@ -776,11 +790,11 @@
       <c r="J3" s="33"/>
     </row>
     <row r="4" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="25"/>
+      <c r="A4" s="28"/>
       <c r="B4" s="8"/>
       <c r="C4" s="2"/>
       <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
+      <c r="E4" s="26"/>
       <c r="F4" s="21"/>
       <c r="G4" s="30"/>
       <c r="H4" s="21"/>
@@ -788,11 +802,11 @@
       <c r="J4" s="33"/>
     </row>
     <row r="5" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="25"/>
+      <c r="A5" s="28"/>
       <c r="B5" s="8"/>
       <c r="C5" s="10"/>
       <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
+      <c r="E5" s="26"/>
       <c r="F5" s="21"/>
       <c r="G5" s="30"/>
       <c r="H5" s="21"/>
@@ -800,11 +814,11 @@
       <c r="J5" s="33"/>
     </row>
     <row r="6" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="25"/>
+      <c r="A6" s="28"/>
       <c r="B6" s="8"/>
       <c r="C6" s="10"/>
       <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
+      <c r="E6" s="26"/>
       <c r="F6" s="21"/>
       <c r="G6" s="30"/>
       <c r="H6" s="21"/>
@@ -812,11 +826,11 @@
       <c r="J6" s="33"/>
     </row>
     <row r="7" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="25"/>
+      <c r="A7" s="28"/>
       <c r="B7" s="9"/>
       <c r="C7" s="10"/>
       <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
+      <c r="E7" s="26"/>
       <c r="F7" s="21"/>
       <c r="G7" s="30"/>
       <c r="H7" s="21"/>
@@ -824,11 +838,11 @@
       <c r="J7" s="33"/>
     </row>
     <row r="8" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="25"/>
+      <c r="A8" s="28"/>
       <c r="B8" s="9"/>
       <c r="C8" s="10"/>
       <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
+      <c r="E8" s="27"/>
       <c r="F8" s="21"/>
       <c r="G8" s="31"/>
       <c r="H8" s="21"/>
@@ -952,10 +966,10 @@
         <v>45915</v>
       </c>
       <c r="C16" s="10"/>
-      <c r="D16" s="26" t="s">
+      <c r="D16" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="E16" s="26" t="s">
+      <c r="E16" s="25" t="s">
         <v>24</v>
       </c>
       <c r="F16" s="21">
@@ -979,8 +993,8 @@
         <v>45916</v>
       </c>
       <c r="C17" s="10"/>
-      <c r="D17" s="27"/>
-      <c r="E17" s="27"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
       <c r="F17" s="21"/>
       <c r="G17" s="30"/>
       <c r="H17" s="21"/>
@@ -994,8 +1008,8 @@
         <v>45917</v>
       </c>
       <c r="C18" s="10"/>
-      <c r="D18" s="27"/>
-      <c r="E18" s="27"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="26"/>
       <c r="F18" s="21"/>
       <c r="G18" s="30"/>
       <c r="H18" s="21"/>
@@ -1009,8 +1023,8 @@
         <v>45918</v>
       </c>
       <c r="C19" s="10"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="27"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
       <c r="F19" s="21"/>
       <c r="G19" s="30"/>
       <c r="H19" s="21"/>
@@ -1024,8 +1038,8 @@
         <v>45919</v>
       </c>
       <c r="C20" s="10"/>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="26"/>
       <c r="F20" s="21"/>
       <c r="G20" s="30"/>
       <c r="H20" s="21"/>
@@ -1039,8 +1053,8 @@
         <v>45920</v>
       </c>
       <c r="C21" s="10"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="27"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="26"/>
       <c r="F21" s="21"/>
       <c r="G21" s="30"/>
       <c r="H21" s="21"/>
@@ -1054,8 +1068,8 @@
         <v>45921</v>
       </c>
       <c r="C22" s="10"/>
-      <c r="D22" s="28"/>
-      <c r="E22" s="28"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="27"/>
       <c r="F22" s="21"/>
       <c r="G22" s="31"/>
       <c r="H22" s="21"/>
@@ -1071,10 +1085,10 @@
         <v>45922</v>
       </c>
       <c r="C23" s="10"/>
-      <c r="D23" s="26" t="s">
+      <c r="D23" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E23" s="26" t="s">
+      <c r="E23" s="25" t="s">
         <v>25</v>
       </c>
       <c r="F23" s="21">
@@ -1098,8 +1112,8 @@
         <v>45923</v>
       </c>
       <c r="C24" s="10"/>
-      <c r="D24" s="27"/>
-      <c r="E24" s="27"/>
+      <c r="D24" s="26"/>
+      <c r="E24" s="26"/>
       <c r="F24" s="21"/>
       <c r="G24" s="30"/>
       <c r="H24" s="21"/>
@@ -1113,8 +1127,8 @@
         <v>45924</v>
       </c>
       <c r="C25" s="10"/>
-      <c r="D25" s="27"/>
-      <c r="E25" s="27"/>
+      <c r="D25" s="26"/>
+      <c r="E25" s="26"/>
       <c r="F25" s="21"/>
       <c r="G25" s="30"/>
       <c r="H25" s="21"/>
@@ -1128,8 +1142,8 @@
         <v>45925</v>
       </c>
       <c r="C26" s="10"/>
-      <c r="D26" s="27"/>
-      <c r="E26" s="27"/>
+      <c r="D26" s="26"/>
+      <c r="E26" s="26"/>
       <c r="F26" s="21"/>
       <c r="G26" s="30"/>
       <c r="H26" s="21"/>
@@ -1143,8 +1157,8 @@
         <v>45926</v>
       </c>
       <c r="C27" s="10"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="27"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
       <c r="F27" s="21"/>
       <c r="G27" s="30"/>
       <c r="H27" s="21"/>
@@ -1158,8 +1172,8 @@
         <v>45927</v>
       </c>
       <c r="C28" s="10"/>
-      <c r="D28" s="27"/>
-      <c r="E28" s="27"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="26"/>
       <c r="F28" s="21"/>
       <c r="G28" s="30"/>
       <c r="H28" s="21"/>
@@ -1173,8 +1187,8 @@
         <v>45928</v>
       </c>
       <c r="C29" s="10"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="27"/>
       <c r="F29" s="21"/>
       <c r="G29" s="31"/>
       <c r="H29" s="21"/>
@@ -1190,10 +1204,10 @@
         <v>45929</v>
       </c>
       <c r="C30" s="10"/>
-      <c r="D30" s="26" t="s">
+      <c r="D30" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E30" s="26" t="s">
+      <c r="E30" s="25" t="s">
         <v>33</v>
       </c>
       <c r="F30" s="21">
@@ -1217,8 +1231,8 @@
         <v>45930</v>
       </c>
       <c r="C31" s="10"/>
-      <c r="D31" s="27"/>
-      <c r="E31" s="27"/>
+      <c r="D31" s="26"/>
+      <c r="E31" s="26"/>
       <c r="F31" s="21"/>
       <c r="G31" s="30"/>
       <c r="H31" s="21"/>
@@ -1234,8 +1248,8 @@
       <c r="C32" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D32" s="27"/>
-      <c r="E32" s="27"/>
+      <c r="D32" s="26"/>
+      <c r="E32" s="26"/>
       <c r="F32" s="21"/>
       <c r="G32" s="30"/>
       <c r="H32" s="21"/>
@@ -1249,8 +1263,8 @@
         <v>45932</v>
       </c>
       <c r="C33" s="10"/>
-      <c r="D33" s="27"/>
-      <c r="E33" s="27"/>
+      <c r="D33" s="26"/>
+      <c r="E33" s="26"/>
       <c r="F33" s="21"/>
       <c r="G33" s="30"/>
       <c r="H33" s="21"/>
@@ -1264,8 +1278,8 @@
         <v>45933</v>
       </c>
       <c r="C34" s="10"/>
-      <c r="D34" s="27"/>
-      <c r="E34" s="27"/>
+      <c r="D34" s="26"/>
+      <c r="E34" s="26"/>
       <c r="F34" s="21"/>
       <c r="G34" s="30"/>
       <c r="H34" s="21"/>
@@ -1279,8 +1293,8 @@
         <v>45934</v>
       </c>
       <c r="C35" s="10"/>
-      <c r="D35" s="27"/>
-      <c r="E35" s="27"/>
+      <c r="D35" s="26"/>
+      <c r="E35" s="26"/>
       <c r="F35" s="21"/>
       <c r="G35" s="30"/>
       <c r="H35" s="21"/>
@@ -1294,8 +1308,8 @@
         <v>45935</v>
       </c>
       <c r="C36" s="10"/>
-      <c r="D36" s="28"/>
-      <c r="E36" s="28"/>
+      <c r="D36" s="27"/>
+      <c r="E36" s="27"/>
       <c r="F36" s="21"/>
       <c r="G36" s="31"/>
       <c r="H36" s="21"/>
@@ -1314,7 +1328,7 @@
       <c r="D37" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="E37" s="22" t="s">
+      <c r="E37" s="25" t="s">
         <v>32</v>
       </c>
       <c r="F37" s="21">
@@ -1341,7 +1355,7 @@
       <c r="D38" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="E38" s="23"/>
+      <c r="E38" s="26"/>
       <c r="F38" s="21"/>
       <c r="G38" s="30"/>
       <c r="H38" s="21"/>
@@ -1356,7 +1370,7 @@
       </c>
       <c r="C39" s="10"/>
       <c r="D39" s="23"/>
-      <c r="E39" s="23"/>
+      <c r="E39" s="26"/>
       <c r="F39" s="21"/>
       <c r="G39" s="30"/>
       <c r="H39" s="21"/>
@@ -1373,7 +1387,7 @@
         <v>8</v>
       </c>
       <c r="D40" s="23"/>
-      <c r="E40" s="23"/>
+      <c r="E40" s="26"/>
       <c r="F40" s="21"/>
       <c r="G40" s="30"/>
       <c r="H40" s="21"/>
@@ -1388,7 +1402,7 @@
       </c>
       <c r="C41" s="10"/>
       <c r="D41" s="23"/>
-      <c r="E41" s="23"/>
+      <c r="E41" s="26"/>
       <c r="F41" s="21"/>
       <c r="G41" s="30"/>
       <c r="H41" s="21"/>
@@ -1403,7 +1417,7 @@
       </c>
       <c r="C42" s="10"/>
       <c r="D42" s="23"/>
-      <c r="E42" s="23"/>
+      <c r="E42" s="26"/>
       <c r="F42" s="21"/>
       <c r="G42" s="30"/>
       <c r="H42" s="21"/>
@@ -1418,7 +1432,7 @@
       </c>
       <c r="C43" s="10"/>
       <c r="D43" s="24"/>
-      <c r="E43" s="24"/>
+      <c r="E43" s="27"/>
       <c r="F43" s="21"/>
       <c r="G43" s="31"/>
       <c r="H43" s="21"/>
@@ -1437,7 +1451,7 @@
       <c r="D44" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="E44" s="38" t="s">
+      <c r="E44" s="25" t="s">
         <v>34</v>
       </c>
       <c r="F44" s="21">
@@ -1464,7 +1478,7 @@
         <v>9</v>
       </c>
       <c r="D45" s="23"/>
-      <c r="E45" s="39"/>
+      <c r="E45" s="26"/>
       <c r="F45" s="21"/>
       <c r="G45" s="30"/>
       <c r="H45" s="21"/>
@@ -1479,7 +1493,7 @@
       </c>
       <c r="C46" s="10"/>
       <c r="D46" s="23"/>
-      <c r="E46" s="39"/>
+      <c r="E46" s="26"/>
       <c r="F46" s="21"/>
       <c r="G46" s="30"/>
       <c r="H46" s="21"/>
@@ -1494,7 +1508,7 @@
       </c>
       <c r="C47" s="10"/>
       <c r="D47" s="23"/>
-      <c r="E47" s="39"/>
+      <c r="E47" s="26"/>
       <c r="F47" s="21"/>
       <c r="G47" s="30"/>
       <c r="H47" s="21"/>
@@ -1509,7 +1523,7 @@
       </c>
       <c r="C48" s="10"/>
       <c r="D48" s="23"/>
-      <c r="E48" s="39"/>
+      <c r="E48" s="26"/>
       <c r="F48" s="21"/>
       <c r="G48" s="30"/>
       <c r="H48" s="21"/>
@@ -1524,7 +1538,7 @@
       </c>
       <c r="C49" s="10"/>
       <c r="D49" s="23"/>
-      <c r="E49" s="39"/>
+      <c r="E49" s="26"/>
       <c r="F49" s="21"/>
       <c r="G49" s="30"/>
       <c r="H49" s="21"/>
@@ -1539,7 +1553,7 @@
       </c>
       <c r="C50" s="10"/>
       <c r="D50" s="24"/>
-      <c r="E50" s="40"/>
+      <c r="E50" s="27"/>
       <c r="F50" s="21"/>
       <c r="G50" s="31"/>
       <c r="H50" s="21"/>
@@ -1558,7 +1572,7 @@
       <c r="D51" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="E51" s="38" t="s">
+      <c r="E51" s="25" t="s">
         <v>35</v>
       </c>
       <c r="F51" s="21">
@@ -1583,7 +1597,7 @@
       </c>
       <c r="C52" s="10"/>
       <c r="D52" s="23"/>
-      <c r="E52" s="39"/>
+      <c r="E52" s="26"/>
       <c r="F52" s="21"/>
       <c r="G52" s="30"/>
       <c r="H52" s="21"/>
@@ -1598,7 +1612,7 @@
       </c>
       <c r="C53" s="10"/>
       <c r="D53" s="23"/>
-      <c r="E53" s="39"/>
+      <c r="E53" s="26"/>
       <c r="F53" s="21"/>
       <c r="G53" s="30"/>
       <c r="H53" s="21"/>
@@ -1613,7 +1627,7 @@
       </c>
       <c r="C54" s="10"/>
       <c r="D54" s="23"/>
-      <c r="E54" s="39"/>
+      <c r="E54" s="26"/>
       <c r="F54" s="21"/>
       <c r="G54" s="30"/>
       <c r="H54" s="21"/>
@@ -1628,7 +1642,7 @@
       </c>
       <c r="C55" s="10"/>
       <c r="D55" s="23"/>
-      <c r="E55" s="39"/>
+      <c r="E55" s="26"/>
       <c r="F55" s="21"/>
       <c r="G55" s="30"/>
       <c r="H55" s="21"/>
@@ -1643,7 +1657,7 @@
       </c>
       <c r="C56" s="12"/>
       <c r="D56" s="23"/>
-      <c r="E56" s="39"/>
+      <c r="E56" s="26"/>
       <c r="F56" s="21"/>
       <c r="G56" s="30"/>
       <c r="H56" s="21"/>
@@ -1658,7 +1672,7 @@
       </c>
       <c r="C57" s="12"/>
       <c r="D57" s="24"/>
-      <c r="E57" s="40"/>
+      <c r="E57" s="27"/>
       <c r="F57" s="21"/>
       <c r="G57" s="31"/>
       <c r="H57" s="21"/>
@@ -1675,9 +1689,11 @@
       </c>
       <c r="C58" s="12"/>
       <c r="D58" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="E58" s="38"/>
+        <v>36</v>
+      </c>
+      <c r="E58" s="25" t="s">
+        <v>37</v>
+      </c>
       <c r="F58" s="21">
         <v>6</v>
       </c>
@@ -1688,7 +1704,7 @@
         <v>6</v>
       </c>
       <c r="I58" s="29">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J58" s="32"/>
     </row>
@@ -1700,7 +1716,7 @@
       </c>
       <c r="C59" s="12"/>
       <c r="D59" s="23"/>
-      <c r="E59" s="39"/>
+      <c r="E59" s="26"/>
       <c r="F59" s="21"/>
       <c r="G59" s="30"/>
       <c r="H59" s="21"/>
@@ -1715,7 +1731,7 @@
       </c>
       <c r="C60" s="12"/>
       <c r="D60" s="23"/>
-      <c r="E60" s="39"/>
+      <c r="E60" s="26"/>
       <c r="F60" s="21"/>
       <c r="G60" s="30"/>
       <c r="H60" s="21"/>
@@ -1730,7 +1746,7 @@
       </c>
       <c r="C61" s="12"/>
       <c r="D61" s="23"/>
-      <c r="E61" s="39"/>
+      <c r="E61" s="26"/>
       <c r="F61" s="21"/>
       <c r="G61" s="30"/>
       <c r="H61" s="21"/>
@@ -1745,7 +1761,7 @@
       </c>
       <c r="C62" s="12"/>
       <c r="D62" s="23"/>
-      <c r="E62" s="39"/>
+      <c r="E62" s="26"/>
       <c r="F62" s="21"/>
       <c r="G62" s="30"/>
       <c r="H62" s="21"/>
@@ -1760,7 +1776,7 @@
       </c>
       <c r="C63" s="12"/>
       <c r="D63" s="23"/>
-      <c r="E63" s="39"/>
+      <c r="E63" s="26"/>
       <c r="F63" s="21"/>
       <c r="G63" s="30"/>
       <c r="H63" s="21"/>
@@ -1775,7 +1791,7 @@
       </c>
       <c r="C64" s="12"/>
       <c r="D64" s="24"/>
-      <c r="E64" s="40"/>
+      <c r="E64" s="27"/>
       <c r="F64" s="21"/>
       <c r="G64" s="31"/>
       <c r="H64" s="21"/>
@@ -1792,17 +1808,23 @@
       </c>
       <c r="C65" s="10"/>
       <c r="D65" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="E65" s="38"/>
+        <v>36</v>
+      </c>
+      <c r="E65" s="25" t="s">
+        <v>38</v>
+      </c>
       <c r="F65" s="21">
         <v>6</v>
       </c>
-      <c r="G65" s="35"/>
+      <c r="G65" s="29">
+        <v>6</v>
+      </c>
       <c r="H65" s="21">
         <v>6</v>
       </c>
-      <c r="I65" s="35"/>
+      <c r="I65" s="29">
+        <v>1</v>
+      </c>
       <c r="J65" s="32"/>
     </row>
     <row r="66" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -1813,11 +1835,11 @@
       </c>
       <c r="C66" s="10"/>
       <c r="D66" s="23"/>
-      <c r="E66" s="39"/>
+      <c r="E66" s="26"/>
       <c r="F66" s="21"/>
-      <c r="G66" s="36"/>
+      <c r="G66" s="30"/>
       <c r="H66" s="21"/>
-      <c r="I66" s="36"/>
+      <c r="I66" s="30"/>
       <c r="J66" s="33"/>
     </row>
     <row r="67" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -1828,11 +1850,11 @@
       </c>
       <c r="C67" s="10"/>
       <c r="D67" s="23"/>
-      <c r="E67" s="39"/>
+      <c r="E67" s="26"/>
       <c r="F67" s="21"/>
-      <c r="G67" s="36"/>
+      <c r="G67" s="30"/>
       <c r="H67" s="21"/>
-      <c r="I67" s="36"/>
+      <c r="I67" s="30"/>
       <c r="J67" s="33"/>
     </row>
     <row r="68" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -1843,11 +1865,11 @@
       </c>
       <c r="C68" s="10"/>
       <c r="D68" s="23"/>
-      <c r="E68" s="39"/>
+      <c r="E68" s="26"/>
       <c r="F68" s="21"/>
-      <c r="G68" s="36"/>
+      <c r="G68" s="30"/>
       <c r="H68" s="21"/>
-      <c r="I68" s="36"/>
+      <c r="I68" s="30"/>
       <c r="J68" s="33"/>
     </row>
     <row r="69" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -1858,11 +1880,11 @@
       </c>
       <c r="C69" s="10"/>
       <c r="D69" s="23"/>
-      <c r="E69" s="39"/>
+      <c r="E69" s="26"/>
       <c r="F69" s="21"/>
-      <c r="G69" s="36"/>
+      <c r="G69" s="30"/>
       <c r="H69" s="21"/>
-      <c r="I69" s="36"/>
+      <c r="I69" s="30"/>
       <c r="J69" s="33"/>
     </row>
     <row r="70" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -1873,11 +1895,11 @@
       </c>
       <c r="C70" s="10"/>
       <c r="D70" s="23"/>
-      <c r="E70" s="39"/>
+      <c r="E70" s="26"/>
       <c r="F70" s="21"/>
-      <c r="G70" s="36"/>
+      <c r="G70" s="30"/>
       <c r="H70" s="21"/>
-      <c r="I70" s="36"/>
+      <c r="I70" s="30"/>
       <c r="J70" s="33"/>
     </row>
     <row r="71" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -1888,11 +1910,11 @@
       </c>
       <c r="C71" s="10"/>
       <c r="D71" s="24"/>
-      <c r="E71" s="40"/>
+      <c r="E71" s="27"/>
       <c r="F71" s="21"/>
-      <c r="G71" s="37"/>
+      <c r="G71" s="31"/>
       <c r="H71" s="21"/>
-      <c r="I71" s="37"/>
+      <c r="I71" s="31"/>
       <c r="J71" s="34"/>
     </row>
     <row r="72" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -1905,17 +1927,23 @@
       </c>
       <c r="C72" s="10"/>
       <c r="D72" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="E72" s="38"/>
+        <v>36</v>
+      </c>
+      <c r="E72" s="35" t="s">
+        <v>40</v>
+      </c>
       <c r="F72" s="21">
         <v>6</v>
       </c>
-      <c r="G72" s="35"/>
+      <c r="G72" s="29">
+        <v>6</v>
+      </c>
       <c r="H72" s="21">
         <v>6</v>
       </c>
-      <c r="I72" s="35"/>
+      <c r="I72" s="29">
+        <v>6</v>
+      </c>
       <c r="J72" s="32"/>
     </row>
     <row r="73" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -1926,11 +1954,11 @@
       </c>
       <c r="C73" s="10"/>
       <c r="D73" s="23"/>
-      <c r="E73" s="39"/>
+      <c r="E73" s="36"/>
       <c r="F73" s="21"/>
-      <c r="G73" s="36"/>
+      <c r="G73" s="30"/>
       <c r="H73" s="21"/>
-      <c r="I73" s="36"/>
+      <c r="I73" s="30"/>
       <c r="J73" s="33"/>
     </row>
     <row r="74" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -1941,11 +1969,11 @@
       </c>
       <c r="C74" s="10"/>
       <c r="D74" s="23"/>
-      <c r="E74" s="39"/>
+      <c r="E74" s="36"/>
       <c r="F74" s="21"/>
-      <c r="G74" s="36"/>
+      <c r="G74" s="30"/>
       <c r="H74" s="21"/>
-      <c r="I74" s="36"/>
+      <c r="I74" s="30"/>
       <c r="J74" s="33"/>
     </row>
     <row r="75" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -1956,11 +1984,11 @@
       </c>
       <c r="C75" s="10"/>
       <c r="D75" s="23"/>
-      <c r="E75" s="39"/>
+      <c r="E75" s="36"/>
       <c r="F75" s="21"/>
-      <c r="G75" s="36"/>
+      <c r="G75" s="30"/>
       <c r="H75" s="21"/>
-      <c r="I75" s="36"/>
+      <c r="I75" s="30"/>
       <c r="J75" s="33"/>
     </row>
     <row r="76" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -1971,11 +1999,11 @@
       </c>
       <c r="C76" s="10"/>
       <c r="D76" s="23"/>
-      <c r="E76" s="39"/>
+      <c r="E76" s="36"/>
       <c r="F76" s="21"/>
-      <c r="G76" s="36"/>
+      <c r="G76" s="30"/>
       <c r="H76" s="21"/>
-      <c r="I76" s="36"/>
+      <c r="I76" s="30"/>
       <c r="J76" s="33"/>
     </row>
     <row r="77" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -1986,11 +2014,11 @@
       </c>
       <c r="C77" s="10"/>
       <c r="D77" s="23"/>
-      <c r="E77" s="39"/>
+      <c r="E77" s="36"/>
       <c r="F77" s="21"/>
-      <c r="G77" s="36"/>
+      <c r="G77" s="30"/>
       <c r="H77" s="21"/>
-      <c r="I77" s="36"/>
+      <c r="I77" s="30"/>
       <c r="J77" s="33"/>
     </row>
     <row r="78" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2001,11 +2029,11 @@
       </c>
       <c r="C78" s="10"/>
       <c r="D78" s="24"/>
-      <c r="E78" s="40"/>
+      <c r="E78" s="37"/>
       <c r="F78" s="21"/>
-      <c r="G78" s="37"/>
+      <c r="G78" s="31"/>
       <c r="H78" s="21"/>
-      <c r="I78" s="37"/>
+      <c r="I78" s="31"/>
       <c r="J78" s="34"/>
     </row>
     <row r="79" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2018,17 +2046,23 @@
       </c>
       <c r="C79" s="10"/>
       <c r="D79" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="E79" s="38"/>
+        <v>36</v>
+      </c>
+      <c r="E79" s="35" t="s">
+        <v>41</v>
+      </c>
       <c r="F79" s="21">
         <v>6</v>
       </c>
-      <c r="G79" s="35"/>
+      <c r="G79" s="29">
+        <v>6</v>
+      </c>
       <c r="H79" s="21">
         <v>6</v>
       </c>
-      <c r="I79" s="35"/>
+      <c r="I79" s="29">
+        <v>6</v>
+      </c>
       <c r="J79" s="32"/>
     </row>
     <row r="80" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2039,11 +2073,11 @@
       </c>
       <c r="C80" s="10"/>
       <c r="D80" s="23"/>
-      <c r="E80" s="39"/>
+      <c r="E80" s="36"/>
       <c r="F80" s="21"/>
-      <c r="G80" s="36"/>
+      <c r="G80" s="30"/>
       <c r="H80" s="21"/>
-      <c r="I80" s="36"/>
+      <c r="I80" s="30"/>
       <c r="J80" s="33"/>
     </row>
     <row r="81" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2054,11 +2088,11 @@
       </c>
       <c r="C81" s="10"/>
       <c r="D81" s="23"/>
-      <c r="E81" s="39"/>
+      <c r="E81" s="36"/>
       <c r="F81" s="21"/>
-      <c r="G81" s="36"/>
+      <c r="G81" s="30"/>
       <c r="H81" s="21"/>
-      <c r="I81" s="36"/>
+      <c r="I81" s="30"/>
       <c r="J81" s="33"/>
     </row>
     <row r="82" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2069,11 +2103,11 @@
       </c>
       <c r="C82" s="10"/>
       <c r="D82" s="23"/>
-      <c r="E82" s="39"/>
+      <c r="E82" s="36"/>
       <c r="F82" s="21"/>
-      <c r="G82" s="36"/>
+      <c r="G82" s="30"/>
       <c r="H82" s="21"/>
-      <c r="I82" s="36"/>
+      <c r="I82" s="30"/>
       <c r="J82" s="33"/>
     </row>
     <row r="83" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2084,11 +2118,11 @@
       </c>
       <c r="C83" s="10"/>
       <c r="D83" s="23"/>
-      <c r="E83" s="39"/>
+      <c r="E83" s="36"/>
       <c r="F83" s="21"/>
-      <c r="G83" s="36"/>
+      <c r="G83" s="30"/>
       <c r="H83" s="21"/>
-      <c r="I83" s="36"/>
+      <c r="I83" s="30"/>
       <c r="J83" s="33"/>
     </row>
     <row r="84" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2099,11 +2133,11 @@
       </c>
       <c r="C84" s="10"/>
       <c r="D84" s="23"/>
-      <c r="E84" s="39"/>
+      <c r="E84" s="36"/>
       <c r="F84" s="21"/>
-      <c r="G84" s="36"/>
+      <c r="G84" s="30"/>
       <c r="H84" s="21"/>
-      <c r="I84" s="36"/>
+      <c r="I84" s="30"/>
       <c r="J84" s="33"/>
     </row>
     <row r="85" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2114,11 +2148,11 @@
       </c>
       <c r="C85" s="10"/>
       <c r="D85" s="24"/>
-      <c r="E85" s="40"/>
+      <c r="E85" s="37"/>
       <c r="F85" s="21"/>
-      <c r="G85" s="37"/>
+      <c r="G85" s="31"/>
       <c r="H85" s="21"/>
-      <c r="I85" s="37"/>
+      <c r="I85" s="31"/>
       <c r="J85" s="34"/>
     </row>
     <row r="86" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2133,15 +2167,21 @@
       <c r="D86" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="E86" s="38"/>
+      <c r="E86" s="35" t="s">
+        <v>39</v>
+      </c>
       <c r="F86" s="21">
         <v>6</v>
       </c>
-      <c r="G86" s="35"/>
+      <c r="G86" s="29">
+        <v>6</v>
+      </c>
       <c r="H86" s="21">
         <v>6</v>
       </c>
-      <c r="I86" s="35"/>
+      <c r="I86" s="29">
+        <v>6</v>
+      </c>
       <c r="J86" s="32"/>
     </row>
     <row r="87" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2152,11 +2192,11 @@
       </c>
       <c r="C87" s="10"/>
       <c r="D87" s="23"/>
-      <c r="E87" s="39"/>
+      <c r="E87" s="36"/>
       <c r="F87" s="21"/>
-      <c r="G87" s="36"/>
+      <c r="G87" s="30"/>
       <c r="H87" s="21"/>
-      <c r="I87" s="36"/>
+      <c r="I87" s="30"/>
       <c r="J87" s="33"/>
     </row>
     <row r="88" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2167,11 +2207,11 @@
       </c>
       <c r="C88" s="10"/>
       <c r="D88" s="23"/>
-      <c r="E88" s="39"/>
+      <c r="E88" s="36"/>
       <c r="F88" s="21"/>
-      <c r="G88" s="36"/>
+      <c r="G88" s="30"/>
       <c r="H88" s="21"/>
-      <c r="I88" s="36"/>
+      <c r="I88" s="30"/>
       <c r="J88" s="33"/>
     </row>
     <row r="89" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2182,11 +2222,11 @@
       </c>
       <c r="C89" s="10"/>
       <c r="D89" s="23"/>
-      <c r="E89" s="39"/>
+      <c r="E89" s="36"/>
       <c r="F89" s="21"/>
-      <c r="G89" s="36"/>
+      <c r="G89" s="30"/>
       <c r="H89" s="21"/>
-      <c r="I89" s="36"/>
+      <c r="I89" s="30"/>
       <c r="J89" s="33"/>
     </row>
     <row r="90" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2197,11 +2237,11 @@
       </c>
       <c r="C90" s="10"/>
       <c r="D90" s="23"/>
-      <c r="E90" s="39"/>
+      <c r="E90" s="36"/>
       <c r="F90" s="21"/>
-      <c r="G90" s="36"/>
+      <c r="G90" s="30"/>
       <c r="H90" s="21"/>
-      <c r="I90" s="36"/>
+      <c r="I90" s="30"/>
       <c r="J90" s="33"/>
     </row>
     <row r="91" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2212,11 +2252,11 @@
       </c>
       <c r="C91" s="10"/>
       <c r="D91" s="23"/>
-      <c r="E91" s="39"/>
+      <c r="E91" s="36"/>
       <c r="F91" s="21"/>
-      <c r="G91" s="36"/>
+      <c r="G91" s="30"/>
       <c r="H91" s="21"/>
-      <c r="I91" s="36"/>
+      <c r="I91" s="30"/>
       <c r="J91" s="33"/>
     </row>
     <row r="92" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2227,11 +2267,11 @@
       </c>
       <c r="C92" s="10"/>
       <c r="D92" s="24"/>
-      <c r="E92" s="40"/>
+      <c r="E92" s="37"/>
       <c r="F92" s="21"/>
-      <c r="G92" s="37"/>
+      <c r="G92" s="31"/>
       <c r="H92" s="21"/>
-      <c r="I92" s="37"/>
+      <c r="I92" s="31"/>
       <c r="J92" s="34"/>
     </row>
     <row r="93" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2246,15 +2286,15 @@
       <c r="D93" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="E93" s="38"/>
+      <c r="E93" s="35"/>
       <c r="F93" s="21">
         <v>6</v>
       </c>
-      <c r="G93" s="35"/>
+      <c r="G93" s="38"/>
       <c r="H93" s="21">
         <v>6</v>
       </c>
-      <c r="I93" s="35"/>
+      <c r="I93" s="38"/>
       <c r="J93" s="32"/>
     </row>
     <row r="94" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2265,11 +2305,11 @@
       </c>
       <c r="C94" s="10"/>
       <c r="D94" s="23"/>
-      <c r="E94" s="39"/>
+      <c r="E94" s="36"/>
       <c r="F94" s="21"/>
-      <c r="G94" s="36"/>
+      <c r="G94" s="39"/>
       <c r="H94" s="21"/>
-      <c r="I94" s="36"/>
+      <c r="I94" s="39"/>
       <c r="J94" s="33"/>
     </row>
     <row r="95" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2280,11 +2320,11 @@
       </c>
       <c r="C95" s="10"/>
       <c r="D95" s="23"/>
-      <c r="E95" s="39"/>
+      <c r="E95" s="36"/>
       <c r="F95" s="21"/>
-      <c r="G95" s="36"/>
+      <c r="G95" s="39"/>
       <c r="H95" s="21"/>
-      <c r="I95" s="36"/>
+      <c r="I95" s="39"/>
       <c r="J95" s="33"/>
     </row>
     <row r="96" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2295,11 +2335,11 @@
       </c>
       <c r="C96" s="10"/>
       <c r="D96" s="23"/>
-      <c r="E96" s="39"/>
+      <c r="E96" s="36"/>
       <c r="F96" s="21"/>
-      <c r="G96" s="36"/>
+      <c r="G96" s="39"/>
       <c r="H96" s="21"/>
-      <c r="I96" s="36"/>
+      <c r="I96" s="39"/>
       <c r="J96" s="33"/>
     </row>
     <row r="97" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2312,11 +2352,11 @@
         <v>10</v>
       </c>
       <c r="D97" s="23"/>
-      <c r="E97" s="39"/>
+      <c r="E97" s="36"/>
       <c r="F97" s="21"/>
-      <c r="G97" s="36"/>
+      <c r="G97" s="39"/>
       <c r="H97" s="21"/>
-      <c r="I97" s="36"/>
+      <c r="I97" s="39"/>
       <c r="J97" s="33"/>
     </row>
     <row r="98" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2327,11 +2367,11 @@
       </c>
       <c r="C98" s="10"/>
       <c r="D98" s="23"/>
-      <c r="E98" s="39"/>
+      <c r="E98" s="36"/>
       <c r="F98" s="21"/>
-      <c r="G98" s="36"/>
+      <c r="G98" s="39"/>
       <c r="H98" s="21"/>
-      <c r="I98" s="36"/>
+      <c r="I98" s="39"/>
       <c r="J98" s="33"/>
     </row>
     <row r="99" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2342,11 +2382,11 @@
       </c>
       <c r="C99" s="10"/>
       <c r="D99" s="24"/>
-      <c r="E99" s="40"/>
+      <c r="E99" s="37"/>
       <c r="F99" s="21"/>
-      <c r="G99" s="37"/>
+      <c r="G99" s="40"/>
       <c r="H99" s="21"/>
-      <c r="I99" s="37"/>
+      <c r="I99" s="40"/>
       <c r="J99" s="34"/>
     </row>
     <row r="100" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2361,15 +2401,15 @@
       <c r="D100" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="E100" s="38"/>
+      <c r="E100" s="35"/>
       <c r="F100" s="21">
         <v>6</v>
       </c>
-      <c r="G100" s="35"/>
+      <c r="G100" s="38"/>
       <c r="H100" s="21">
         <v>6</v>
       </c>
-      <c r="I100" s="35"/>
+      <c r="I100" s="38"/>
       <c r="J100" s="32"/>
     </row>
     <row r="101" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2380,11 +2420,11 @@
       </c>
       <c r="C101" s="10"/>
       <c r="D101" s="23"/>
-      <c r="E101" s="39"/>
+      <c r="E101" s="36"/>
       <c r="F101" s="21"/>
-      <c r="G101" s="36"/>
+      <c r="G101" s="39"/>
       <c r="H101" s="21"/>
-      <c r="I101" s="36"/>
+      <c r="I101" s="39"/>
       <c r="J101" s="33"/>
     </row>
     <row r="102" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2395,11 +2435,11 @@
       </c>
       <c r="C102" s="10"/>
       <c r="D102" s="23"/>
-      <c r="E102" s="39"/>
+      <c r="E102" s="36"/>
       <c r="F102" s="21"/>
-      <c r="G102" s="36"/>
+      <c r="G102" s="39"/>
       <c r="H102" s="21"/>
-      <c r="I102" s="36"/>
+      <c r="I102" s="39"/>
       <c r="J102" s="33"/>
     </row>
     <row r="103" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2410,11 +2450,11 @@
       </c>
       <c r="C103" s="10"/>
       <c r="D103" s="23"/>
-      <c r="E103" s="39"/>
+      <c r="E103" s="36"/>
       <c r="F103" s="21"/>
-      <c r="G103" s="36"/>
+      <c r="G103" s="39"/>
       <c r="H103" s="21"/>
-      <c r="I103" s="36"/>
+      <c r="I103" s="39"/>
       <c r="J103" s="33"/>
     </row>
     <row r="104" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2425,11 +2465,11 @@
       </c>
       <c r="C104" s="10"/>
       <c r="D104" s="23"/>
-      <c r="E104" s="39"/>
+      <c r="E104" s="36"/>
       <c r="F104" s="21"/>
-      <c r="G104" s="36"/>
+      <c r="G104" s="39"/>
       <c r="H104" s="21"/>
-      <c r="I104" s="36"/>
+      <c r="I104" s="39"/>
       <c r="J104" s="33"/>
     </row>
     <row r="105" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2440,11 +2480,11 @@
       </c>
       <c r="C105" s="10"/>
       <c r="D105" s="23"/>
-      <c r="E105" s="39"/>
+      <c r="E105" s="36"/>
       <c r="F105" s="21"/>
-      <c r="G105" s="36"/>
+      <c r="G105" s="39"/>
       <c r="H105" s="21"/>
-      <c r="I105" s="36"/>
+      <c r="I105" s="39"/>
       <c r="J105" s="33"/>
     </row>
     <row r="106" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2455,11 +2495,11 @@
       </c>
       <c r="C106" s="10"/>
       <c r="D106" s="24"/>
-      <c r="E106" s="40"/>
+      <c r="E106" s="37"/>
       <c r="F106" s="21"/>
-      <c r="G106" s="37"/>
+      <c r="G106" s="40"/>
       <c r="H106" s="21"/>
-      <c r="I106" s="37"/>
+      <c r="I106" s="40"/>
       <c r="J106" s="34"/>
     </row>
     <row r="107" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2474,15 +2514,15 @@
       <c r="D107" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="E107" s="38"/>
+      <c r="E107" s="35"/>
       <c r="F107" s="21">
         <v>6</v>
       </c>
-      <c r="G107" s="35"/>
+      <c r="G107" s="38"/>
       <c r="H107" s="21">
         <v>6</v>
       </c>
-      <c r="I107" s="35"/>
+      <c r="I107" s="38"/>
       <c r="J107" s="32"/>
     </row>
     <row r="108" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2493,11 +2533,11 @@
       </c>
       <c r="C108" s="10"/>
       <c r="D108" s="23"/>
-      <c r="E108" s="39"/>
+      <c r="E108" s="36"/>
       <c r="F108" s="21"/>
-      <c r="G108" s="36"/>
+      <c r="G108" s="39"/>
       <c r="H108" s="21"/>
-      <c r="I108" s="36"/>
+      <c r="I108" s="39"/>
       <c r="J108" s="33"/>
     </row>
     <row r="109" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2508,11 +2548,11 @@
       </c>
       <c r="C109" s="10"/>
       <c r="D109" s="23"/>
-      <c r="E109" s="39"/>
+      <c r="E109" s="36"/>
       <c r="F109" s="21"/>
-      <c r="G109" s="36"/>
+      <c r="G109" s="39"/>
       <c r="H109" s="21"/>
-      <c r="I109" s="36"/>
+      <c r="I109" s="39"/>
       <c r="J109" s="33"/>
     </row>
     <row r="110" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2523,11 +2563,11 @@
       </c>
       <c r="C110" s="10"/>
       <c r="D110" s="23"/>
-      <c r="E110" s="39"/>
+      <c r="E110" s="36"/>
       <c r="F110" s="21"/>
-      <c r="G110" s="36"/>
+      <c r="G110" s="39"/>
       <c r="H110" s="21"/>
-      <c r="I110" s="36"/>
+      <c r="I110" s="39"/>
       <c r="J110" s="33"/>
     </row>
     <row r="111" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2538,11 +2578,11 @@
       </c>
       <c r="C111" s="10"/>
       <c r="D111" s="23"/>
-      <c r="E111" s="39"/>
+      <c r="E111" s="36"/>
       <c r="F111" s="21"/>
-      <c r="G111" s="36"/>
+      <c r="G111" s="39"/>
       <c r="H111" s="21"/>
-      <c r="I111" s="36"/>
+      <c r="I111" s="39"/>
       <c r="J111" s="33"/>
     </row>
     <row r="112" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2553,11 +2593,11 @@
       </c>
       <c r="C112" s="10"/>
       <c r="D112" s="23"/>
-      <c r="E112" s="39"/>
+      <c r="E112" s="36"/>
       <c r="F112" s="21"/>
-      <c r="G112" s="36"/>
+      <c r="G112" s="39"/>
       <c r="H112" s="21"/>
-      <c r="I112" s="36"/>
+      <c r="I112" s="39"/>
       <c r="J112" s="33"/>
     </row>
     <row r="113" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2568,11 +2608,11 @@
       </c>
       <c r="C113" s="10"/>
       <c r="D113" s="24"/>
-      <c r="E113" s="40"/>
+      <c r="E113" s="37"/>
       <c r="F113" s="21"/>
-      <c r="G113" s="37"/>
+      <c r="G113" s="40"/>
       <c r="H113" s="21"/>
-      <c r="I113" s="37"/>
+      <c r="I113" s="40"/>
       <c r="J113" s="34"/>
     </row>
     <row r="114" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2587,15 +2627,15 @@
       <c r="D114" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="E114" s="38"/>
+      <c r="E114" s="35"/>
       <c r="F114" s="21">
         <v>6</v>
       </c>
-      <c r="G114" s="35"/>
+      <c r="G114" s="38"/>
       <c r="H114" s="21">
         <v>6</v>
       </c>
-      <c r="I114" s="35"/>
+      <c r="I114" s="38"/>
       <c r="J114" s="32"/>
     </row>
     <row r="115" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2606,11 +2646,11 @@
       </c>
       <c r="C115" s="10"/>
       <c r="D115" s="23"/>
-      <c r="E115" s="39"/>
+      <c r="E115" s="36"/>
       <c r="F115" s="21"/>
-      <c r="G115" s="36"/>
+      <c r="G115" s="39"/>
       <c r="H115" s="21"/>
-      <c r="I115" s="36"/>
+      <c r="I115" s="39"/>
       <c r="J115" s="33"/>
     </row>
     <row r="116" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2621,11 +2661,11 @@
       </c>
       <c r="C116" s="12"/>
       <c r="D116" s="23"/>
-      <c r="E116" s="39"/>
+      <c r="E116" s="36"/>
       <c r="F116" s="21"/>
-      <c r="G116" s="36"/>
+      <c r="G116" s="39"/>
       <c r="H116" s="21"/>
-      <c r="I116" s="36"/>
+      <c r="I116" s="39"/>
       <c r="J116" s="33"/>
     </row>
     <row r="117" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2636,11 +2676,11 @@
       </c>
       <c r="C117" s="12"/>
       <c r="D117" s="23"/>
-      <c r="E117" s="39"/>
+      <c r="E117" s="36"/>
       <c r="F117" s="21"/>
-      <c r="G117" s="36"/>
+      <c r="G117" s="39"/>
       <c r="H117" s="21"/>
-      <c r="I117" s="36"/>
+      <c r="I117" s="39"/>
       <c r="J117" s="33"/>
     </row>
     <row r="118" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2651,11 +2691,11 @@
       </c>
       <c r="C118" s="12"/>
       <c r="D118" s="23"/>
-      <c r="E118" s="39"/>
+      <c r="E118" s="36"/>
       <c r="F118" s="21"/>
-      <c r="G118" s="36"/>
+      <c r="G118" s="39"/>
       <c r="H118" s="21"/>
-      <c r="I118" s="36"/>
+      <c r="I118" s="39"/>
       <c r="J118" s="33"/>
     </row>
     <row r="119" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2666,11 +2706,11 @@
       </c>
       <c r="C119" s="12"/>
       <c r="D119" s="23"/>
-      <c r="E119" s="39"/>
+      <c r="E119" s="36"/>
       <c r="F119" s="21"/>
-      <c r="G119" s="36"/>
+      <c r="G119" s="39"/>
       <c r="H119" s="21"/>
-      <c r="I119" s="36"/>
+      <c r="I119" s="39"/>
       <c r="J119" s="33"/>
     </row>
     <row r="120" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2681,11 +2721,11 @@
       </c>
       <c r="C120" s="12"/>
       <c r="D120" s="24"/>
-      <c r="E120" s="40"/>
+      <c r="E120" s="37"/>
       <c r="F120" s="21"/>
-      <c r="G120" s="37"/>
+      <c r="G120" s="40"/>
       <c r="H120" s="21"/>
-      <c r="I120" s="37"/>
+      <c r="I120" s="40"/>
       <c r="J120" s="34"/>
     </row>
     <row r="121" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2700,15 +2740,15 @@
       <c r="D121" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="E121" s="38"/>
+      <c r="E121" s="35"/>
       <c r="F121" s="21">
         <v>6</v>
       </c>
-      <c r="G121" s="35"/>
+      <c r="G121" s="38"/>
       <c r="H121" s="21">
         <v>6</v>
       </c>
-      <c r="I121" s="35"/>
+      <c r="I121" s="38"/>
       <c r="J121" s="32"/>
     </row>
     <row r="122" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2719,11 +2759,11 @@
       </c>
       <c r="C122" s="12"/>
       <c r="D122" s="23"/>
-      <c r="E122" s="39"/>
+      <c r="E122" s="36"/>
       <c r="F122" s="21"/>
-      <c r="G122" s="36"/>
+      <c r="G122" s="39"/>
       <c r="H122" s="21"/>
-      <c r="I122" s="36"/>
+      <c r="I122" s="39"/>
       <c r="J122" s="33"/>
     </row>
     <row r="123" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2734,11 +2774,11 @@
       </c>
       <c r="C123" s="12"/>
       <c r="D123" s="23"/>
-      <c r="E123" s="39"/>
+      <c r="E123" s="36"/>
       <c r="F123" s="21"/>
-      <c r="G123" s="36"/>
+      <c r="G123" s="39"/>
       <c r="H123" s="21"/>
-      <c r="I123" s="36"/>
+      <c r="I123" s="39"/>
       <c r="J123" s="33"/>
     </row>
     <row r="124" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2749,11 +2789,11 @@
       </c>
       <c r="C124" s="12"/>
       <c r="D124" s="23"/>
-      <c r="E124" s="39"/>
+      <c r="E124" s="36"/>
       <c r="F124" s="21"/>
-      <c r="G124" s="36"/>
+      <c r="G124" s="39"/>
       <c r="H124" s="21"/>
-      <c r="I124" s="36"/>
+      <c r="I124" s="39"/>
       <c r="J124" s="33"/>
     </row>
     <row r="125" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2764,11 +2804,11 @@
       </c>
       <c r="C125" s="12"/>
       <c r="D125" s="23"/>
-      <c r="E125" s="39"/>
+      <c r="E125" s="36"/>
       <c r="F125" s="21"/>
-      <c r="G125" s="36"/>
+      <c r="G125" s="39"/>
       <c r="H125" s="21"/>
-      <c r="I125" s="36"/>
+      <c r="I125" s="39"/>
       <c r="J125" s="33"/>
     </row>
     <row r="126" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2779,11 +2819,11 @@
       </c>
       <c r="C126" s="12"/>
       <c r="D126" s="23"/>
-      <c r="E126" s="39"/>
+      <c r="E126" s="36"/>
       <c r="F126" s="21"/>
-      <c r="G126" s="36"/>
+      <c r="G126" s="39"/>
       <c r="H126" s="21"/>
-      <c r="I126" s="36"/>
+      <c r="I126" s="39"/>
       <c r="J126" s="33"/>
     </row>
     <row r="127" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2794,11 +2834,11 @@
       </c>
       <c r="C127" s="12"/>
       <c r="D127" s="24"/>
-      <c r="E127" s="40"/>
+      <c r="E127" s="37"/>
       <c r="F127" s="21"/>
-      <c r="G127" s="37"/>
+      <c r="G127" s="40"/>
       <c r="H127" s="21"/>
-      <c r="I127" s="37"/>
+      <c r="I127" s="40"/>
       <c r="J127" s="34"/>
     </row>
     <row r="128" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2813,15 +2853,15 @@
       <c r="D128" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="E128" s="38"/>
+      <c r="E128" s="35"/>
       <c r="F128" s="21">
         <v>6</v>
       </c>
-      <c r="G128" s="35"/>
+      <c r="G128" s="38"/>
       <c r="H128" s="21">
         <v>6</v>
       </c>
-      <c r="I128" s="35"/>
+      <c r="I128" s="38"/>
       <c r="J128" s="32"/>
     </row>
     <row r="129" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2832,11 +2872,11 @@
       </c>
       <c r="C129" s="12"/>
       <c r="D129" s="23"/>
-      <c r="E129" s="39"/>
+      <c r="E129" s="36"/>
       <c r="F129" s="21"/>
-      <c r="G129" s="36"/>
+      <c r="G129" s="39"/>
       <c r="H129" s="21"/>
-      <c r="I129" s="36"/>
+      <c r="I129" s="39"/>
       <c r="J129" s="33"/>
     </row>
     <row r="130" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2847,11 +2887,11 @@
       </c>
       <c r="C130" s="10"/>
       <c r="D130" s="23"/>
-      <c r="E130" s="39"/>
+      <c r="E130" s="36"/>
       <c r="F130" s="21"/>
-      <c r="G130" s="36"/>
+      <c r="G130" s="39"/>
       <c r="H130" s="21"/>
-      <c r="I130" s="36"/>
+      <c r="I130" s="39"/>
       <c r="J130" s="33"/>
     </row>
     <row r="131" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2862,11 +2902,11 @@
       </c>
       <c r="C131" s="10"/>
       <c r="D131" s="23"/>
-      <c r="E131" s="39"/>
+      <c r="E131" s="36"/>
       <c r="F131" s="21"/>
-      <c r="G131" s="36"/>
+      <c r="G131" s="39"/>
       <c r="H131" s="21"/>
-      <c r="I131" s="36"/>
+      <c r="I131" s="39"/>
       <c r="J131" s="33"/>
     </row>
     <row r="132" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2877,11 +2917,11 @@
       </c>
       <c r="C132" s="10"/>
       <c r="D132" s="23"/>
-      <c r="E132" s="39"/>
+      <c r="E132" s="36"/>
       <c r="F132" s="21"/>
-      <c r="G132" s="36"/>
+      <c r="G132" s="39"/>
       <c r="H132" s="21"/>
-      <c r="I132" s="36"/>
+      <c r="I132" s="39"/>
       <c r="J132" s="33"/>
     </row>
     <row r="133" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2892,11 +2932,11 @@
       </c>
       <c r="C133" s="10"/>
       <c r="D133" s="23"/>
-      <c r="E133" s="39"/>
+      <c r="E133" s="36"/>
       <c r="F133" s="21"/>
-      <c r="G133" s="36"/>
+      <c r="G133" s="39"/>
       <c r="H133" s="21"/>
-      <c r="I133" s="36"/>
+      <c r="I133" s="39"/>
       <c r="J133" s="33"/>
     </row>
     <row r="134" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2907,11 +2947,11 @@
       </c>
       <c r="C134" s="10"/>
       <c r="D134" s="24"/>
-      <c r="E134" s="40"/>
+      <c r="E134" s="37"/>
       <c r="F134" s="21"/>
-      <c r="G134" s="37"/>
+      <c r="G134" s="40"/>
       <c r="H134" s="21"/>
-      <c r="I134" s="37"/>
+      <c r="I134" s="40"/>
       <c r="J134" s="34"/>
     </row>
     <row r="135" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2926,15 +2966,15 @@
       <c r="D135" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="E135" s="38"/>
+      <c r="E135" s="35"/>
       <c r="F135" s="21">
         <v>6</v>
       </c>
-      <c r="G135" s="35"/>
+      <c r="G135" s="38"/>
       <c r="H135" s="21">
         <v>6</v>
       </c>
-      <c r="I135" s="35"/>
+      <c r="I135" s="38"/>
       <c r="J135" s="32"/>
     </row>
     <row r="136" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2945,11 +2985,11 @@
       </c>
       <c r="C136" s="10"/>
       <c r="D136" s="23"/>
-      <c r="E136" s="39"/>
+      <c r="E136" s="36"/>
       <c r="F136" s="21"/>
-      <c r="G136" s="36"/>
+      <c r="G136" s="39"/>
       <c r="H136" s="21"/>
-      <c r="I136" s="36"/>
+      <c r="I136" s="39"/>
       <c r="J136" s="33"/>
     </row>
     <row r="137" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2960,11 +3000,11 @@
       </c>
       <c r="C137" s="10"/>
       <c r="D137" s="23"/>
-      <c r="E137" s="39"/>
+      <c r="E137" s="36"/>
       <c r="F137" s="21"/>
-      <c r="G137" s="36"/>
+      <c r="G137" s="39"/>
       <c r="H137" s="21"/>
-      <c r="I137" s="36"/>
+      <c r="I137" s="39"/>
       <c r="J137" s="33"/>
     </row>
     <row r="138" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2975,11 +3015,11 @@
       </c>
       <c r="C138" s="10"/>
       <c r="D138" s="23"/>
-      <c r="E138" s="39"/>
+      <c r="E138" s="36"/>
       <c r="F138" s="21"/>
-      <c r="G138" s="36"/>
+      <c r="G138" s="39"/>
       <c r="H138" s="21"/>
-      <c r="I138" s="36"/>
+      <c r="I138" s="39"/>
       <c r="J138" s="33"/>
     </row>
     <row r="139" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -2990,11 +3030,11 @@
       </c>
       <c r="C139" s="10"/>
       <c r="D139" s="23"/>
-      <c r="E139" s="39"/>
+      <c r="E139" s="36"/>
       <c r="F139" s="21"/>
-      <c r="G139" s="36"/>
+      <c r="G139" s="39"/>
       <c r="H139" s="21"/>
-      <c r="I139" s="36"/>
+      <c r="I139" s="39"/>
       <c r="J139" s="33"/>
     </row>
     <row r="140" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3005,11 +3045,11 @@
       </c>
       <c r="C140" s="10"/>
       <c r="D140" s="23"/>
-      <c r="E140" s="39"/>
+      <c r="E140" s="36"/>
       <c r="F140" s="21"/>
-      <c r="G140" s="36"/>
+      <c r="G140" s="39"/>
       <c r="H140" s="21"/>
-      <c r="I140" s="36"/>
+      <c r="I140" s="39"/>
       <c r="J140" s="33"/>
     </row>
     <row r="141" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3020,11 +3060,11 @@
       </c>
       <c r="C141" s="10"/>
       <c r="D141" s="24"/>
-      <c r="E141" s="40"/>
+      <c r="E141" s="37"/>
       <c r="F141" s="21"/>
-      <c r="G141" s="37"/>
+      <c r="G141" s="40"/>
       <c r="H141" s="21"/>
-      <c r="I141" s="37"/>
+      <c r="I141" s="40"/>
       <c r="J141" s="34"/>
     </row>
     <row r="142" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3039,15 +3079,15 @@
       <c r="D142" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="E142" s="38"/>
+      <c r="E142" s="35"/>
       <c r="F142" s="21">
         <v>6</v>
       </c>
-      <c r="G142" s="35"/>
+      <c r="G142" s="38"/>
       <c r="H142" s="21">
         <v>6</v>
       </c>
-      <c r="I142" s="35"/>
+      <c r="I142" s="38"/>
       <c r="J142" s="32"/>
     </row>
     <row r="143" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3058,11 +3098,11 @@
       </c>
       <c r="C143" s="10"/>
       <c r="D143" s="23"/>
-      <c r="E143" s="39"/>
+      <c r="E143" s="36"/>
       <c r="F143" s="21"/>
-      <c r="G143" s="36"/>
+      <c r="G143" s="39"/>
       <c r="H143" s="21"/>
-      <c r="I143" s="36"/>
+      <c r="I143" s="39"/>
       <c r="J143" s="33"/>
     </row>
     <row r="144" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3073,11 +3113,11 @@
       </c>
       <c r="C144" s="10"/>
       <c r="D144" s="23"/>
-      <c r="E144" s="39"/>
+      <c r="E144" s="36"/>
       <c r="F144" s="21"/>
-      <c r="G144" s="36"/>
+      <c r="G144" s="39"/>
       <c r="H144" s="21"/>
-      <c r="I144" s="36"/>
+      <c r="I144" s="39"/>
       <c r="J144" s="33"/>
     </row>
     <row r="145" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3088,11 +3128,11 @@
       </c>
       <c r="C145" s="10"/>
       <c r="D145" s="23"/>
-      <c r="E145" s="39"/>
+      <c r="E145" s="36"/>
       <c r="F145" s="21"/>
-      <c r="G145" s="36"/>
+      <c r="G145" s="39"/>
       <c r="H145" s="21"/>
-      <c r="I145" s="36"/>
+      <c r="I145" s="39"/>
       <c r="J145" s="33"/>
     </row>
     <row r="146" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3103,11 +3143,11 @@
       </c>
       <c r="C146" s="10"/>
       <c r="D146" s="23"/>
-      <c r="E146" s="39"/>
+      <c r="E146" s="36"/>
       <c r="F146" s="21"/>
-      <c r="G146" s="36"/>
+      <c r="G146" s="39"/>
       <c r="H146" s="21"/>
-      <c r="I146" s="36"/>
+      <c r="I146" s="39"/>
       <c r="J146" s="33"/>
     </row>
     <row r="147" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3118,11 +3158,11 @@
       </c>
       <c r="C147" s="10"/>
       <c r="D147" s="23"/>
-      <c r="E147" s="39"/>
+      <c r="E147" s="36"/>
       <c r="F147" s="21"/>
-      <c r="G147" s="36"/>
+      <c r="G147" s="39"/>
       <c r="H147" s="21"/>
-      <c r="I147" s="36"/>
+      <c r="I147" s="39"/>
       <c r="J147" s="33"/>
     </row>
     <row r="148" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3133,11 +3173,11 @@
       </c>
       <c r="C148" s="10"/>
       <c r="D148" s="24"/>
-      <c r="E148" s="40"/>
+      <c r="E148" s="37"/>
       <c r="F148" s="21"/>
-      <c r="G148" s="37"/>
+      <c r="G148" s="40"/>
       <c r="H148" s="21"/>
-      <c r="I148" s="37"/>
+      <c r="I148" s="40"/>
       <c r="J148" s="34"/>
     </row>
     <row r="149" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3152,15 +3192,15 @@
       <c r="D149" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="E149" s="38"/>
+      <c r="E149" s="35"/>
       <c r="F149" s="21">
         <v>6</v>
       </c>
-      <c r="G149" s="35"/>
+      <c r="G149" s="38"/>
       <c r="H149" s="21">
         <v>6</v>
       </c>
-      <c r="I149" s="35"/>
+      <c r="I149" s="38"/>
       <c r="J149" s="32"/>
     </row>
     <row r="150" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3171,11 +3211,11 @@
       </c>
       <c r="C150" s="10"/>
       <c r="D150" s="23"/>
-      <c r="E150" s="39"/>
+      <c r="E150" s="36"/>
       <c r="F150" s="21"/>
-      <c r="G150" s="36"/>
+      <c r="G150" s="39"/>
       <c r="H150" s="21"/>
-      <c r="I150" s="36"/>
+      <c r="I150" s="39"/>
       <c r="J150" s="33"/>
     </row>
     <row r="151" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3186,11 +3226,11 @@
       </c>
       <c r="C151" s="10"/>
       <c r="D151" s="23"/>
-      <c r="E151" s="39"/>
+      <c r="E151" s="36"/>
       <c r="F151" s="21"/>
-      <c r="G151" s="36"/>
+      <c r="G151" s="39"/>
       <c r="H151" s="21"/>
-      <c r="I151" s="36"/>
+      <c r="I151" s="39"/>
       <c r="J151" s="33"/>
     </row>
     <row r="152" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3201,11 +3241,11 @@
       </c>
       <c r="C152" s="10"/>
       <c r="D152" s="23"/>
-      <c r="E152" s="39"/>
+      <c r="E152" s="36"/>
       <c r="F152" s="21"/>
-      <c r="G152" s="36"/>
+      <c r="G152" s="39"/>
       <c r="H152" s="21"/>
-      <c r="I152" s="36"/>
+      <c r="I152" s="39"/>
       <c r="J152" s="33"/>
     </row>
     <row r="153" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3216,11 +3256,11 @@
       </c>
       <c r="C153" s="10"/>
       <c r="D153" s="23"/>
-      <c r="E153" s="39"/>
+      <c r="E153" s="36"/>
       <c r="F153" s="21"/>
-      <c r="G153" s="36"/>
+      <c r="G153" s="39"/>
       <c r="H153" s="21"/>
-      <c r="I153" s="36"/>
+      <c r="I153" s="39"/>
       <c r="J153" s="33"/>
     </row>
     <row r="154" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3231,11 +3271,11 @@
       </c>
       <c r="C154" s="10"/>
       <c r="D154" s="23"/>
-      <c r="E154" s="39"/>
+      <c r="E154" s="36"/>
       <c r="F154" s="21"/>
-      <c r="G154" s="36"/>
+      <c r="G154" s="39"/>
       <c r="H154" s="21"/>
-      <c r="I154" s="36"/>
+      <c r="I154" s="39"/>
       <c r="J154" s="33"/>
     </row>
     <row r="155" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3246,11 +3286,11 @@
       </c>
       <c r="C155" s="10"/>
       <c r="D155" s="24"/>
-      <c r="E155" s="40"/>
+      <c r="E155" s="37"/>
       <c r="F155" s="21"/>
-      <c r="G155" s="37"/>
+      <c r="G155" s="40"/>
       <c r="H155" s="21"/>
-      <c r="I155" s="37"/>
+      <c r="I155" s="40"/>
       <c r="J155" s="34"/>
     </row>
     <row r="156" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3265,15 +3305,15 @@
       <c r="D156" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="E156" s="38"/>
+      <c r="E156" s="35"/>
       <c r="F156" s="21">
         <v>6</v>
       </c>
-      <c r="G156" s="35"/>
+      <c r="G156" s="38"/>
       <c r="H156" s="21">
         <v>6</v>
       </c>
-      <c r="I156" s="35"/>
+      <c r="I156" s="38"/>
       <c r="J156" s="32"/>
     </row>
     <row r="157" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3284,11 +3324,11 @@
       </c>
       <c r="C157" s="10"/>
       <c r="D157" s="23"/>
-      <c r="E157" s="39"/>
+      <c r="E157" s="36"/>
       <c r="F157" s="21"/>
-      <c r="G157" s="36"/>
+      <c r="G157" s="39"/>
       <c r="H157" s="21"/>
-      <c r="I157" s="36"/>
+      <c r="I157" s="39"/>
       <c r="J157" s="33"/>
     </row>
     <row r="158" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3299,11 +3339,11 @@
       </c>
       <c r="C158" s="10"/>
       <c r="D158" s="23"/>
-      <c r="E158" s="39"/>
+      <c r="E158" s="36"/>
       <c r="F158" s="21"/>
-      <c r="G158" s="36"/>
+      <c r="G158" s="39"/>
       <c r="H158" s="21"/>
-      <c r="I158" s="36"/>
+      <c r="I158" s="39"/>
       <c r="J158" s="33"/>
     </row>
     <row r="159" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3314,11 +3354,11 @@
       </c>
       <c r="C159" s="10"/>
       <c r="D159" s="23"/>
-      <c r="E159" s="39"/>
+      <c r="E159" s="36"/>
       <c r="F159" s="21"/>
-      <c r="G159" s="36"/>
+      <c r="G159" s="39"/>
       <c r="H159" s="21"/>
-      <c r="I159" s="36"/>
+      <c r="I159" s="39"/>
       <c r="J159" s="33"/>
     </row>
     <row r="160" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3329,11 +3369,11 @@
       </c>
       <c r="C160" s="10"/>
       <c r="D160" s="23"/>
-      <c r="E160" s="39"/>
+      <c r="E160" s="36"/>
       <c r="F160" s="21"/>
-      <c r="G160" s="36"/>
+      <c r="G160" s="39"/>
       <c r="H160" s="21"/>
-      <c r="I160" s="36"/>
+      <c r="I160" s="39"/>
       <c r="J160" s="33"/>
     </row>
     <row r="161" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3344,11 +3384,11 @@
       </c>
       <c r="C161" s="10"/>
       <c r="D161" s="23"/>
-      <c r="E161" s="39"/>
+      <c r="E161" s="36"/>
       <c r="F161" s="21"/>
-      <c r="G161" s="36"/>
+      <c r="G161" s="39"/>
       <c r="H161" s="21"/>
-      <c r="I161" s="36"/>
+      <c r="I161" s="39"/>
       <c r="J161" s="33"/>
     </row>
     <row r="162" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3359,11 +3399,11 @@
       </c>
       <c r="C162" s="10"/>
       <c r="D162" s="24"/>
-      <c r="E162" s="40"/>
+      <c r="E162" s="37"/>
       <c r="F162" s="21"/>
-      <c r="G162" s="37"/>
+      <c r="G162" s="40"/>
       <c r="H162" s="21"/>
-      <c r="I162" s="37"/>
+      <c r="I162" s="40"/>
       <c r="J162" s="34"/>
     </row>
     <row r="163" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3380,15 +3420,15 @@
       <c r="D163" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="E163" s="38"/>
+      <c r="E163" s="35"/>
       <c r="F163" s="21">
         <v>6</v>
       </c>
-      <c r="G163" s="35"/>
+      <c r="G163" s="38"/>
       <c r="H163" s="21">
         <v>6</v>
       </c>
-      <c r="I163" s="35"/>
+      <c r="I163" s="38"/>
       <c r="J163" s="32"/>
     </row>
     <row r="164" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3399,11 +3439,11 @@
       </c>
       <c r="C164" s="10"/>
       <c r="D164" s="23"/>
-      <c r="E164" s="39"/>
+      <c r="E164" s="36"/>
       <c r="F164" s="21"/>
-      <c r="G164" s="36"/>
+      <c r="G164" s="39"/>
       <c r="H164" s="21"/>
-      <c r="I164" s="36"/>
+      <c r="I164" s="39"/>
       <c r="J164" s="33"/>
     </row>
     <row r="165" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3414,11 +3454,11 @@
       </c>
       <c r="C165" s="10"/>
       <c r="D165" s="23"/>
-      <c r="E165" s="39"/>
+      <c r="E165" s="36"/>
       <c r="F165" s="21"/>
-      <c r="G165" s="36"/>
+      <c r="G165" s="39"/>
       <c r="H165" s="21"/>
-      <c r="I165" s="36"/>
+      <c r="I165" s="39"/>
       <c r="J165" s="33"/>
     </row>
     <row r="166" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3429,11 +3469,11 @@
       </c>
       <c r="C166" s="10"/>
       <c r="D166" s="23"/>
-      <c r="E166" s="39"/>
+      <c r="E166" s="36"/>
       <c r="F166" s="21"/>
-      <c r="G166" s="36"/>
+      <c r="G166" s="39"/>
       <c r="H166" s="21"/>
-      <c r="I166" s="36"/>
+      <c r="I166" s="39"/>
       <c r="J166" s="33"/>
     </row>
     <row r="167" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3446,11 +3486,11 @@
         <v>12</v>
       </c>
       <c r="D167" s="23"/>
-      <c r="E167" s="39"/>
+      <c r="E167" s="36"/>
       <c r="F167" s="21"/>
-      <c r="G167" s="36"/>
+      <c r="G167" s="39"/>
       <c r="H167" s="21"/>
-      <c r="I167" s="36"/>
+      <c r="I167" s="39"/>
       <c r="J167" s="33"/>
     </row>
     <row r="168" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3461,11 +3501,11 @@
       </c>
       <c r="C168" s="10"/>
       <c r="D168" s="23"/>
-      <c r="E168" s="39"/>
+      <c r="E168" s="36"/>
       <c r="F168" s="21"/>
-      <c r="G168" s="36"/>
+      <c r="G168" s="39"/>
       <c r="H168" s="21"/>
-      <c r="I168" s="36"/>
+      <c r="I168" s="39"/>
       <c r="J168" s="33"/>
     </row>
     <row r="169" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3476,11 +3516,11 @@
       </c>
       <c r="C169" s="10"/>
       <c r="D169" s="24"/>
-      <c r="E169" s="40"/>
+      <c r="E169" s="37"/>
       <c r="F169" s="21"/>
-      <c r="G169" s="37"/>
+      <c r="G169" s="40"/>
       <c r="H169" s="21"/>
-      <c r="I169" s="37"/>
+      <c r="I169" s="40"/>
       <c r="J169" s="34"/>
     </row>
     <row r="170" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3495,15 +3535,15 @@
       <c r="D170" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="E170" s="38"/>
+      <c r="E170" s="35"/>
       <c r="F170" s="21">
         <v>6</v>
       </c>
-      <c r="G170" s="35"/>
+      <c r="G170" s="38"/>
       <c r="H170" s="21">
         <v>6</v>
       </c>
-      <c r="I170" s="35"/>
+      <c r="I170" s="38"/>
       <c r="J170" s="32"/>
     </row>
     <row r="171" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3514,11 +3554,11 @@
       </c>
       <c r="C171" s="12"/>
       <c r="D171" s="23"/>
-      <c r="E171" s="39"/>
+      <c r="E171" s="36"/>
       <c r="F171" s="21"/>
-      <c r="G171" s="36"/>
+      <c r="G171" s="39"/>
       <c r="H171" s="21"/>
-      <c r="I171" s="36"/>
+      <c r="I171" s="39"/>
       <c r="J171" s="33"/>
     </row>
     <row r="172" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3529,11 +3569,11 @@
       </c>
       <c r="C172" s="12"/>
       <c r="D172" s="23"/>
-      <c r="E172" s="39"/>
+      <c r="E172" s="36"/>
       <c r="F172" s="21"/>
-      <c r="G172" s="36"/>
+      <c r="G172" s="39"/>
       <c r="H172" s="21"/>
-      <c r="I172" s="36"/>
+      <c r="I172" s="39"/>
       <c r="J172" s="33"/>
     </row>
     <row r="173" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3544,11 +3584,11 @@
       </c>
       <c r="C173" s="12"/>
       <c r="D173" s="23"/>
-      <c r="E173" s="39"/>
+      <c r="E173" s="36"/>
       <c r="F173" s="21"/>
-      <c r="G173" s="36"/>
+      <c r="G173" s="39"/>
       <c r="H173" s="21"/>
-      <c r="I173" s="36"/>
+      <c r="I173" s="39"/>
       <c r="J173" s="33"/>
     </row>
     <row r="174" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3559,11 +3599,11 @@
       </c>
       <c r="C174" s="12"/>
       <c r="D174" s="23"/>
-      <c r="E174" s="39"/>
+      <c r="E174" s="36"/>
       <c r="F174" s="21"/>
-      <c r="G174" s="36"/>
+      <c r="G174" s="39"/>
       <c r="H174" s="21"/>
-      <c r="I174" s="36"/>
+      <c r="I174" s="39"/>
       <c r="J174" s="33"/>
     </row>
     <row r="175" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3574,11 +3614,11 @@
       </c>
       <c r="C175" s="12"/>
       <c r="D175" s="23"/>
-      <c r="E175" s="39"/>
+      <c r="E175" s="36"/>
       <c r="F175" s="21"/>
-      <c r="G175" s="36"/>
+      <c r="G175" s="39"/>
       <c r="H175" s="21"/>
-      <c r="I175" s="36"/>
+      <c r="I175" s="39"/>
       <c r="J175" s="33"/>
     </row>
     <row r="176" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3589,11 +3629,11 @@
       </c>
       <c r="C176" s="12"/>
       <c r="D176" s="24"/>
-      <c r="E176" s="40"/>
+      <c r="E176" s="37"/>
       <c r="F176" s="21"/>
-      <c r="G176" s="37"/>
+      <c r="G176" s="40"/>
       <c r="H176" s="21"/>
-      <c r="I176" s="37"/>
+      <c r="I176" s="40"/>
       <c r="J176" s="34"/>
     </row>
     <row r="177" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3606,15 +3646,15 @@
       </c>
       <c r="C177" s="10"/>
       <c r="D177" s="22"/>
-      <c r="E177" s="38"/>
+      <c r="E177" s="35"/>
       <c r="F177" s="21">
         <v>6</v>
       </c>
-      <c r="G177" s="35"/>
+      <c r="G177" s="38"/>
       <c r="H177" s="21">
         <v>6</v>
       </c>
-      <c r="I177" s="35"/>
+      <c r="I177" s="38"/>
       <c r="J177" s="32"/>
     </row>
     <row r="178" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3625,11 +3665,11 @@
       </c>
       <c r="C178" s="10"/>
       <c r="D178" s="23"/>
-      <c r="E178" s="39"/>
+      <c r="E178" s="36"/>
       <c r="F178" s="21"/>
-      <c r="G178" s="36"/>
+      <c r="G178" s="39"/>
       <c r="H178" s="21"/>
-      <c r="I178" s="36"/>
+      <c r="I178" s="39"/>
       <c r="J178" s="33"/>
     </row>
     <row r="179" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3640,11 +3680,11 @@
       </c>
       <c r="C179" s="10"/>
       <c r="D179" s="23"/>
-      <c r="E179" s="39"/>
+      <c r="E179" s="36"/>
       <c r="F179" s="21"/>
-      <c r="G179" s="36"/>
+      <c r="G179" s="39"/>
       <c r="H179" s="21"/>
-      <c r="I179" s="36"/>
+      <c r="I179" s="39"/>
       <c r="J179" s="33"/>
     </row>
     <row r="180" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3655,11 +3695,11 @@
       </c>
       <c r="C180" s="10"/>
       <c r="D180" s="23"/>
-      <c r="E180" s="39"/>
+      <c r="E180" s="36"/>
       <c r="F180" s="21"/>
-      <c r="G180" s="36"/>
+      <c r="G180" s="39"/>
       <c r="H180" s="21"/>
-      <c r="I180" s="36"/>
+      <c r="I180" s="39"/>
       <c r="J180" s="33"/>
     </row>
     <row r="181" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3670,11 +3710,11 @@
       </c>
       <c r="C181" s="10"/>
       <c r="D181" s="23"/>
-      <c r="E181" s="39"/>
+      <c r="E181" s="36"/>
       <c r="F181" s="21"/>
-      <c r="G181" s="36"/>
+      <c r="G181" s="39"/>
       <c r="H181" s="21"/>
-      <c r="I181" s="36"/>
+      <c r="I181" s="39"/>
       <c r="J181" s="33"/>
     </row>
     <row r="182" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3685,11 +3725,11 @@
       </c>
       <c r="C182" s="10"/>
       <c r="D182" s="23"/>
-      <c r="E182" s="39"/>
+      <c r="E182" s="36"/>
       <c r="F182" s="21"/>
-      <c r="G182" s="36"/>
+      <c r="G182" s="39"/>
       <c r="H182" s="21"/>
-      <c r="I182" s="36"/>
+      <c r="I182" s="39"/>
       <c r="J182" s="33"/>
     </row>
     <row r="183" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3700,11 +3740,11 @@
       </c>
       <c r="C183" s="10"/>
       <c r="D183" s="24"/>
-      <c r="E183" s="40"/>
+      <c r="E183" s="37"/>
       <c r="F183" s="21"/>
-      <c r="G183" s="37"/>
+      <c r="G183" s="40"/>
       <c r="H183" s="21"/>
-      <c r="I183" s="37"/>
+      <c r="I183" s="40"/>
       <c r="J183" s="34"/>
     </row>
     <row r="184" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3717,15 +3757,15 @@
       </c>
       <c r="C184" s="10"/>
       <c r="D184" s="22"/>
-      <c r="E184" s="38"/>
+      <c r="E184" s="35"/>
       <c r="F184" s="21">
         <v>6</v>
       </c>
-      <c r="G184" s="35"/>
+      <c r="G184" s="38"/>
       <c r="H184" s="21">
         <v>6</v>
       </c>
-      <c r="I184" s="35"/>
+      <c r="I184" s="38"/>
       <c r="J184" s="32"/>
     </row>
     <row r="185" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3736,11 +3776,11 @@
       </c>
       <c r="C185" s="10"/>
       <c r="D185" s="23"/>
-      <c r="E185" s="39"/>
+      <c r="E185" s="36"/>
       <c r="F185" s="21"/>
-      <c r="G185" s="36"/>
+      <c r="G185" s="39"/>
       <c r="H185" s="21"/>
-      <c r="I185" s="36"/>
+      <c r="I185" s="39"/>
       <c r="J185" s="33"/>
     </row>
     <row r="186" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3751,11 +3791,11 @@
       </c>
       <c r="C186" s="10"/>
       <c r="D186" s="23"/>
-      <c r="E186" s="39"/>
+      <c r="E186" s="36"/>
       <c r="F186" s="21"/>
-      <c r="G186" s="36"/>
+      <c r="G186" s="39"/>
       <c r="H186" s="21"/>
-      <c r="I186" s="36"/>
+      <c r="I186" s="39"/>
       <c r="J186" s="33"/>
     </row>
     <row r="187" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3766,11 +3806,11 @@
       </c>
       <c r="C187" s="10"/>
       <c r="D187" s="23"/>
-      <c r="E187" s="39"/>
+      <c r="E187" s="36"/>
       <c r="F187" s="21"/>
-      <c r="G187" s="36"/>
+      <c r="G187" s="39"/>
       <c r="H187" s="21"/>
-      <c r="I187" s="36"/>
+      <c r="I187" s="39"/>
       <c r="J187" s="33"/>
     </row>
     <row r="188" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3781,11 +3821,11 @@
       </c>
       <c r="C188" s="10"/>
       <c r="D188" s="23"/>
-      <c r="E188" s="39"/>
+      <c r="E188" s="36"/>
       <c r="F188" s="21"/>
-      <c r="G188" s="36"/>
+      <c r="G188" s="39"/>
       <c r="H188" s="21"/>
-      <c r="I188" s="36"/>
+      <c r="I188" s="39"/>
       <c r="J188" s="33"/>
     </row>
     <row r="189" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3796,11 +3836,11 @@
       </c>
       <c r="C189" s="10"/>
       <c r="D189" s="23"/>
-      <c r="E189" s="39"/>
+      <c r="E189" s="36"/>
       <c r="F189" s="21"/>
-      <c r="G189" s="36"/>
+      <c r="G189" s="39"/>
       <c r="H189" s="21"/>
-      <c r="I189" s="36"/>
+      <c r="I189" s="39"/>
       <c r="J189" s="33"/>
     </row>
     <row r="190" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3811,11 +3851,11 @@
       </c>
       <c r="C190" s="10"/>
       <c r="D190" s="24"/>
-      <c r="E190" s="40"/>
+      <c r="E190" s="37"/>
       <c r="F190" s="21"/>
-      <c r="G190" s="37"/>
+      <c r="G190" s="40"/>
       <c r="H190" s="21"/>
-      <c r="I190" s="37"/>
+      <c r="I190" s="40"/>
       <c r="J190" s="34"/>
     </row>
     <row r="191" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3828,15 +3868,15 @@
       </c>
       <c r="C191" s="10"/>
       <c r="D191" s="22"/>
-      <c r="E191" s="38"/>
+      <c r="E191" s="35"/>
       <c r="F191" s="21">
         <v>6</v>
       </c>
-      <c r="G191" s="35"/>
+      <c r="G191" s="38"/>
       <c r="H191" s="21">
         <v>6</v>
       </c>
-      <c r="I191" s="35"/>
+      <c r="I191" s="38"/>
       <c r="J191" s="32"/>
     </row>
     <row r="192" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3849,11 +3889,11 @@
         <v>13</v>
       </c>
       <c r="D192" s="23"/>
-      <c r="E192" s="39"/>
+      <c r="E192" s="36"/>
       <c r="F192" s="21"/>
-      <c r="G192" s="36"/>
+      <c r="G192" s="39"/>
       <c r="H192" s="21"/>
-      <c r="I192" s="36"/>
+      <c r="I192" s="39"/>
       <c r="J192" s="33"/>
     </row>
     <row r="193" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3864,11 +3904,11 @@
       </c>
       <c r="C193" s="10"/>
       <c r="D193" s="23"/>
-      <c r="E193" s="39"/>
+      <c r="E193" s="36"/>
       <c r="F193" s="21"/>
-      <c r="G193" s="36"/>
+      <c r="G193" s="39"/>
       <c r="H193" s="21"/>
-      <c r="I193" s="36"/>
+      <c r="I193" s="39"/>
       <c r="J193" s="33"/>
     </row>
     <row r="194" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3878,11 +3918,11 @@
         <v>46093</v>
       </c>
       <c r="D194" s="23"/>
-      <c r="E194" s="39"/>
+      <c r="E194" s="36"/>
       <c r="F194" s="21"/>
-      <c r="G194" s="36"/>
+      <c r="G194" s="39"/>
       <c r="H194" s="21"/>
-      <c r="I194" s="36"/>
+      <c r="I194" s="39"/>
       <c r="J194" s="33"/>
     </row>
     <row r="195" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3893,11 +3933,11 @@
       </c>
       <c r="C195" s="10"/>
       <c r="D195" s="23"/>
-      <c r="E195" s="39"/>
+      <c r="E195" s="36"/>
       <c r="F195" s="21"/>
-      <c r="G195" s="36"/>
+      <c r="G195" s="39"/>
       <c r="H195" s="21"/>
-      <c r="I195" s="36"/>
+      <c r="I195" s="39"/>
       <c r="J195" s="33"/>
     </row>
     <row r="196" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3908,11 +3948,11 @@
       </c>
       <c r="C196" s="10"/>
       <c r="D196" s="23"/>
-      <c r="E196" s="39"/>
+      <c r="E196" s="36"/>
       <c r="F196" s="21"/>
-      <c r="G196" s="36"/>
+      <c r="G196" s="39"/>
       <c r="H196" s="21"/>
-      <c r="I196" s="36"/>
+      <c r="I196" s="39"/>
       <c r="J196" s="33"/>
     </row>
     <row r="197" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3923,11 +3963,11 @@
       </c>
       <c r="C197" s="10"/>
       <c r="D197" s="24"/>
-      <c r="E197" s="40"/>
+      <c r="E197" s="37"/>
       <c r="F197" s="21"/>
-      <c r="G197" s="37"/>
+      <c r="G197" s="40"/>
       <c r="H197" s="21"/>
-      <c r="I197" s="37"/>
+      <c r="I197" s="40"/>
       <c r="J197" s="34"/>
     </row>
     <row r="198" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3940,15 +3980,15 @@
       </c>
       <c r="C198" s="10"/>
       <c r="D198" s="22"/>
-      <c r="E198" s="38"/>
+      <c r="E198" s="35"/>
       <c r="F198" s="21">
         <v>6</v>
       </c>
-      <c r="G198" s="35"/>
+      <c r="G198" s="38"/>
       <c r="H198" s="21">
         <v>6</v>
       </c>
-      <c r="I198" s="35"/>
+      <c r="I198" s="38"/>
       <c r="J198" s="32"/>
     </row>
     <row r="199" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3959,11 +3999,11 @@
       </c>
       <c r="C199" s="10"/>
       <c r="D199" s="23"/>
-      <c r="E199" s="39"/>
+      <c r="E199" s="36"/>
       <c r="F199" s="21"/>
-      <c r="G199" s="36"/>
+      <c r="G199" s="39"/>
       <c r="H199" s="21"/>
-      <c r="I199" s="36"/>
+      <c r="I199" s="39"/>
       <c r="J199" s="33"/>
     </row>
     <row r="200" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3974,11 +4014,11 @@
       </c>
       <c r="C200" s="10"/>
       <c r="D200" s="23"/>
-      <c r="E200" s="39"/>
+      <c r="E200" s="36"/>
       <c r="F200" s="21"/>
-      <c r="G200" s="36"/>
+      <c r="G200" s="39"/>
       <c r="H200" s="21"/>
-      <c r="I200" s="36"/>
+      <c r="I200" s="39"/>
       <c r="J200" s="33"/>
     </row>
     <row r="201" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -3989,11 +4029,11 @@
       </c>
       <c r="C201" s="10"/>
       <c r="D201" s="23"/>
-      <c r="E201" s="39"/>
+      <c r="E201" s="36"/>
       <c r="F201" s="21"/>
-      <c r="G201" s="36"/>
+      <c r="G201" s="39"/>
       <c r="H201" s="21"/>
-      <c r="I201" s="36"/>
+      <c r="I201" s="39"/>
       <c r="J201" s="33"/>
     </row>
     <row r="202" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4004,11 +4044,11 @@
       </c>
       <c r="C202" s="10"/>
       <c r="D202" s="23"/>
-      <c r="E202" s="39"/>
+      <c r="E202" s="36"/>
       <c r="F202" s="21"/>
-      <c r="G202" s="36"/>
+      <c r="G202" s="39"/>
       <c r="H202" s="21"/>
-      <c r="I202" s="36"/>
+      <c r="I202" s="39"/>
       <c r="J202" s="33"/>
     </row>
     <row r="203" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4019,11 +4059,11 @@
       </c>
       <c r="C203" s="10"/>
       <c r="D203" s="23"/>
-      <c r="E203" s="39"/>
+      <c r="E203" s="36"/>
       <c r="F203" s="21"/>
-      <c r="G203" s="36"/>
+      <c r="G203" s="39"/>
       <c r="H203" s="21"/>
-      <c r="I203" s="36"/>
+      <c r="I203" s="39"/>
       <c r="J203" s="33"/>
     </row>
     <row r="204" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4034,11 +4074,11 @@
       </c>
       <c r="C204" s="10"/>
       <c r="D204" s="24"/>
-      <c r="E204" s="40"/>
+      <c r="E204" s="37"/>
       <c r="F204" s="21"/>
-      <c r="G204" s="37"/>
+      <c r="G204" s="40"/>
       <c r="H204" s="21"/>
-      <c r="I204" s="37"/>
+      <c r="I204" s="40"/>
       <c r="J204" s="34"/>
     </row>
     <row r="205" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4051,15 +4091,15 @@
       </c>
       <c r="C205" s="10"/>
       <c r="D205" s="22"/>
-      <c r="E205" s="38"/>
+      <c r="E205" s="35"/>
       <c r="F205" s="21">
         <v>6</v>
       </c>
-      <c r="G205" s="35"/>
+      <c r="G205" s="38"/>
       <c r="H205" s="21">
         <v>6</v>
       </c>
-      <c r="I205" s="35"/>
+      <c r="I205" s="38"/>
       <c r="J205" s="32"/>
     </row>
     <row r="206" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4070,11 +4110,11 @@
       </c>
       <c r="C206" s="10"/>
       <c r="D206" s="23"/>
-      <c r="E206" s="39"/>
+      <c r="E206" s="36"/>
       <c r="F206" s="21"/>
-      <c r="G206" s="36"/>
+      <c r="G206" s="39"/>
       <c r="H206" s="21"/>
-      <c r="I206" s="36"/>
+      <c r="I206" s="39"/>
       <c r="J206" s="33"/>
     </row>
     <row r="207" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4085,11 +4125,11 @@
       </c>
       <c r="C207" s="10"/>
       <c r="D207" s="23"/>
-      <c r="E207" s="39"/>
+      <c r="E207" s="36"/>
       <c r="F207" s="21"/>
-      <c r="G207" s="36"/>
+      <c r="G207" s="39"/>
       <c r="H207" s="21"/>
-      <c r="I207" s="36"/>
+      <c r="I207" s="39"/>
       <c r="J207" s="33"/>
     </row>
     <row r="208" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4100,11 +4140,11 @@
       </c>
       <c r="C208" s="10"/>
       <c r="D208" s="23"/>
-      <c r="E208" s="39"/>
+      <c r="E208" s="36"/>
       <c r="F208" s="21"/>
-      <c r="G208" s="36"/>
+      <c r="G208" s="39"/>
       <c r="H208" s="21"/>
-      <c r="I208" s="36"/>
+      <c r="I208" s="39"/>
       <c r="J208" s="33"/>
     </row>
     <row r="209" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4115,11 +4155,11 @@
       </c>
       <c r="C209" s="10"/>
       <c r="D209" s="23"/>
-      <c r="E209" s="39"/>
+      <c r="E209" s="36"/>
       <c r="F209" s="21"/>
-      <c r="G209" s="36"/>
+      <c r="G209" s="39"/>
       <c r="H209" s="21"/>
-      <c r="I209" s="36"/>
+      <c r="I209" s="39"/>
       <c r="J209" s="33"/>
     </row>
     <row r="210" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4130,11 +4170,11 @@
       </c>
       <c r="C210" s="10"/>
       <c r="D210" s="23"/>
-      <c r="E210" s="39"/>
+      <c r="E210" s="36"/>
       <c r="F210" s="21"/>
-      <c r="G210" s="36"/>
+      <c r="G210" s="39"/>
       <c r="H210" s="21"/>
-      <c r="I210" s="36"/>
+      <c r="I210" s="39"/>
       <c r="J210" s="33"/>
     </row>
     <row r="211" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4145,11 +4185,11 @@
       </c>
       <c r="C211" s="10"/>
       <c r="D211" s="24"/>
-      <c r="E211" s="40"/>
+      <c r="E211" s="37"/>
       <c r="F211" s="21"/>
-      <c r="G211" s="37"/>
+      <c r="G211" s="40"/>
       <c r="H211" s="21"/>
-      <c r="I211" s="37"/>
+      <c r="I211" s="40"/>
       <c r="J211" s="34"/>
     </row>
     <row r="212" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4162,11 +4202,11 @@
       </c>
       <c r="C212" s="10"/>
       <c r="D212" s="22"/>
-      <c r="E212" s="38"/>
+      <c r="E212" s="35"/>
       <c r="F212" s="21"/>
-      <c r="G212" s="35"/>
-      <c r="H212" s="35"/>
-      <c r="I212" s="35"/>
+      <c r="G212" s="38"/>
+      <c r="H212" s="38"/>
+      <c r="I212" s="38"/>
       <c r="J212" s="32"/>
     </row>
     <row r="213" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4177,11 +4217,11 @@
       </c>
       <c r="C213" s="10"/>
       <c r="D213" s="23"/>
-      <c r="E213" s="39"/>
+      <c r="E213" s="36"/>
       <c r="F213" s="21"/>
-      <c r="G213" s="36"/>
-      <c r="H213" s="36"/>
-      <c r="I213" s="36"/>
+      <c r="G213" s="39"/>
+      <c r="H213" s="39"/>
+      <c r="I213" s="39"/>
       <c r="J213" s="33"/>
     </row>
     <row r="214" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4192,11 +4232,11 @@
       </c>
       <c r="C214" s="10"/>
       <c r="D214" s="23"/>
-      <c r="E214" s="39"/>
+      <c r="E214" s="36"/>
       <c r="F214" s="21"/>
-      <c r="G214" s="36"/>
-      <c r="H214" s="36"/>
-      <c r="I214" s="36"/>
+      <c r="G214" s="39"/>
+      <c r="H214" s="39"/>
+      <c r="I214" s="39"/>
       <c r="J214" s="33"/>
     </row>
     <row r="215" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4207,11 +4247,11 @@
       </c>
       <c r="C215" s="10"/>
       <c r="D215" s="23"/>
-      <c r="E215" s="39"/>
+      <c r="E215" s="36"/>
       <c r="F215" s="21"/>
-      <c r="G215" s="36"/>
-      <c r="H215" s="36"/>
-      <c r="I215" s="36"/>
+      <c r="G215" s="39"/>
+      <c r="H215" s="39"/>
+      <c r="I215" s="39"/>
       <c r="J215" s="33"/>
     </row>
     <row r="216" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4222,11 +4262,11 @@
       </c>
       <c r="C216" s="10"/>
       <c r="D216" s="23"/>
-      <c r="E216" s="39"/>
+      <c r="E216" s="36"/>
       <c r="F216" s="21"/>
-      <c r="G216" s="36"/>
-      <c r="H216" s="36"/>
-      <c r="I216" s="36"/>
+      <c r="G216" s="39"/>
+      <c r="H216" s="39"/>
+      <c r="I216" s="39"/>
       <c r="J216" s="33"/>
     </row>
     <row r="217" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4237,11 +4277,11 @@
       </c>
       <c r="C217" s="10"/>
       <c r="D217" s="23"/>
-      <c r="E217" s="39"/>
+      <c r="E217" s="36"/>
       <c r="F217" s="21"/>
-      <c r="G217" s="36"/>
-      <c r="H217" s="36"/>
-      <c r="I217" s="36"/>
+      <c r="G217" s="39"/>
+      <c r="H217" s="39"/>
+      <c r="I217" s="39"/>
       <c r="J217" s="33"/>
     </row>
     <row r="218" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4252,11 +4292,11 @@
       </c>
       <c r="C218" s="10"/>
       <c r="D218" s="24"/>
-      <c r="E218" s="40"/>
+      <c r="E218" s="37"/>
       <c r="F218" s="21"/>
-      <c r="G218" s="37"/>
-      <c r="H218" s="37"/>
-      <c r="I218" s="37"/>
+      <c r="G218" s="40"/>
+      <c r="H218" s="40"/>
+      <c r="I218" s="40"/>
       <c r="J218" s="34"/>
     </row>
     <row r="219" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4269,11 +4309,11 @@
       </c>
       <c r="C219" s="12"/>
       <c r="D219" s="22"/>
-      <c r="E219" s="38"/>
+      <c r="E219" s="35"/>
       <c r="F219" s="21"/>
-      <c r="G219" s="35"/>
-      <c r="H219" s="35"/>
-      <c r="I219" s="35"/>
+      <c r="G219" s="38"/>
+      <c r="H219" s="38"/>
+      <c r="I219" s="38"/>
       <c r="J219" s="32"/>
     </row>
     <row r="220" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4284,11 +4324,11 @@
       </c>
       <c r="C220" s="12"/>
       <c r="D220" s="23"/>
-      <c r="E220" s="39"/>
+      <c r="E220" s="36"/>
       <c r="F220" s="21"/>
-      <c r="G220" s="36"/>
-      <c r="H220" s="36"/>
-      <c r="I220" s="36"/>
+      <c r="G220" s="39"/>
+      <c r="H220" s="39"/>
+      <c r="I220" s="39"/>
       <c r="J220" s="33"/>
     </row>
     <row r="221" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4299,11 +4339,11 @@
       </c>
       <c r="C221" s="12"/>
       <c r="D221" s="23"/>
-      <c r="E221" s="39"/>
+      <c r="E221" s="36"/>
       <c r="F221" s="21"/>
-      <c r="G221" s="36"/>
-      <c r="H221" s="36"/>
-      <c r="I221" s="36"/>
+      <c r="G221" s="39"/>
+      <c r="H221" s="39"/>
+      <c r="I221" s="39"/>
       <c r="J221" s="33"/>
     </row>
     <row r="222" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4314,11 +4354,11 @@
       </c>
       <c r="C222" s="12"/>
       <c r="D222" s="23"/>
-      <c r="E222" s="39"/>
+      <c r="E222" s="36"/>
       <c r="F222" s="21"/>
-      <c r="G222" s="36"/>
-      <c r="H222" s="36"/>
-      <c r="I222" s="36"/>
+      <c r="G222" s="39"/>
+      <c r="H222" s="39"/>
+      <c r="I222" s="39"/>
       <c r="J222" s="33"/>
     </row>
     <row r="223" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4329,11 +4369,11 @@
       </c>
       <c r="C223" s="12"/>
       <c r="D223" s="23"/>
-      <c r="E223" s="39"/>
+      <c r="E223" s="36"/>
       <c r="F223" s="21"/>
-      <c r="G223" s="36"/>
-      <c r="H223" s="36"/>
-      <c r="I223" s="36"/>
+      <c r="G223" s="39"/>
+      <c r="H223" s="39"/>
+      <c r="I223" s="39"/>
       <c r="J223" s="33"/>
     </row>
     <row r="224" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4344,11 +4384,11 @@
       </c>
       <c r="C224" s="12"/>
       <c r="D224" s="23"/>
-      <c r="E224" s="39"/>
+      <c r="E224" s="36"/>
       <c r="F224" s="21"/>
-      <c r="G224" s="36"/>
-      <c r="H224" s="36"/>
-      <c r="I224" s="36"/>
+      <c r="G224" s="39"/>
+      <c r="H224" s="39"/>
+      <c r="I224" s="39"/>
       <c r="J224" s="33"/>
     </row>
     <row r="225" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4359,11 +4399,11 @@
       </c>
       <c r="C225" s="12"/>
       <c r="D225" s="24"/>
-      <c r="E225" s="40"/>
+      <c r="E225" s="37"/>
       <c r="F225" s="21"/>
-      <c r="G225" s="37"/>
-      <c r="H225" s="37"/>
-      <c r="I225" s="37"/>
+      <c r="G225" s="40"/>
+      <c r="H225" s="40"/>
+      <c r="I225" s="40"/>
       <c r="J225" s="34"/>
     </row>
     <row r="226" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4376,11 +4416,11 @@
       </c>
       <c r="C226" s="12"/>
       <c r="D226" s="22"/>
-      <c r="E226" s="38"/>
+      <c r="E226" s="35"/>
       <c r="F226" s="21"/>
-      <c r="G226" s="35"/>
-      <c r="H226" s="35"/>
-      <c r="I226" s="35"/>
+      <c r="G226" s="38"/>
+      <c r="H226" s="38"/>
+      <c r="I226" s="38"/>
       <c r="J226" s="32"/>
     </row>
     <row r="227" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4391,11 +4431,11 @@
       </c>
       <c r="C227" s="10"/>
       <c r="D227" s="23"/>
-      <c r="E227" s="39"/>
+      <c r="E227" s="36"/>
       <c r="F227" s="21"/>
-      <c r="G227" s="36"/>
-      <c r="H227" s="36"/>
-      <c r="I227" s="36"/>
+      <c r="G227" s="39"/>
+      <c r="H227" s="39"/>
+      <c r="I227" s="39"/>
       <c r="J227" s="33"/>
     </row>
     <row r="228" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4406,11 +4446,11 @@
       </c>
       <c r="C228" s="10"/>
       <c r="D228" s="23"/>
-      <c r="E228" s="39"/>
+      <c r="E228" s="36"/>
       <c r="F228" s="21"/>
-      <c r="G228" s="36"/>
-      <c r="H228" s="36"/>
-      <c r="I228" s="36"/>
+      <c r="G228" s="39"/>
+      <c r="H228" s="39"/>
+      <c r="I228" s="39"/>
       <c r="J228" s="33"/>
     </row>
     <row r="229" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4421,11 +4461,11 @@
       </c>
       <c r="C229" s="10"/>
       <c r="D229" s="23"/>
-      <c r="E229" s="39"/>
+      <c r="E229" s="36"/>
       <c r="F229" s="21"/>
-      <c r="G229" s="36"/>
-      <c r="H229" s="36"/>
-      <c r="I229" s="36"/>
+      <c r="G229" s="39"/>
+      <c r="H229" s="39"/>
+      <c r="I229" s="39"/>
       <c r="J229" s="33"/>
     </row>
     <row r="230" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4436,11 +4476,11 @@
       </c>
       <c r="C230" s="10"/>
       <c r="D230" s="23"/>
-      <c r="E230" s="39"/>
+      <c r="E230" s="36"/>
       <c r="F230" s="21"/>
-      <c r="G230" s="36"/>
-      <c r="H230" s="36"/>
-      <c r="I230" s="36"/>
+      <c r="G230" s="39"/>
+      <c r="H230" s="39"/>
+      <c r="I230" s="39"/>
       <c r="J230" s="33"/>
     </row>
     <row r="231" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4451,11 +4491,11 @@
       </c>
       <c r="C231" s="10"/>
       <c r="D231" s="23"/>
-      <c r="E231" s="39"/>
+      <c r="E231" s="36"/>
       <c r="F231" s="21"/>
-      <c r="G231" s="36"/>
-      <c r="H231" s="36"/>
-      <c r="I231" s="36"/>
+      <c r="G231" s="39"/>
+      <c r="H231" s="39"/>
+      <c r="I231" s="39"/>
       <c r="J231" s="33"/>
     </row>
     <row r="232" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4466,11 +4506,11 @@
       </c>
       <c r="C232" s="10"/>
       <c r="D232" s="24"/>
-      <c r="E232" s="40"/>
+      <c r="E232" s="37"/>
       <c r="F232" s="21"/>
-      <c r="G232" s="37"/>
-      <c r="H232" s="37"/>
-      <c r="I232" s="37"/>
+      <c r="G232" s="40"/>
+      <c r="H232" s="40"/>
+      <c r="I232" s="40"/>
       <c r="J232" s="34"/>
     </row>
     <row r="233" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4483,11 +4523,11 @@
       </c>
       <c r="C233" s="10"/>
       <c r="D233" s="22"/>
-      <c r="E233" s="38"/>
+      <c r="E233" s="35"/>
       <c r="F233" s="21"/>
-      <c r="G233" s="35"/>
-      <c r="H233" s="35"/>
-      <c r="I233" s="35"/>
+      <c r="G233" s="38"/>
+      <c r="H233" s="38"/>
+      <c r="I233" s="38"/>
       <c r="J233" s="32"/>
     </row>
     <row r="234" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4498,11 +4538,11 @@
       </c>
       <c r="C234" s="10"/>
       <c r="D234" s="23"/>
-      <c r="E234" s="39"/>
+      <c r="E234" s="36"/>
       <c r="F234" s="21"/>
-      <c r="G234" s="36"/>
-      <c r="H234" s="36"/>
-      <c r="I234" s="36"/>
+      <c r="G234" s="39"/>
+      <c r="H234" s="39"/>
+      <c r="I234" s="39"/>
       <c r="J234" s="33"/>
     </row>
     <row r="235" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4513,11 +4553,11 @@
       </c>
       <c r="C235" s="10"/>
       <c r="D235" s="23"/>
-      <c r="E235" s="39"/>
+      <c r="E235" s="36"/>
       <c r="F235" s="21"/>
-      <c r="G235" s="36"/>
-      <c r="H235" s="36"/>
-      <c r="I235" s="36"/>
+      <c r="G235" s="39"/>
+      <c r="H235" s="39"/>
+      <c r="I235" s="39"/>
       <c r="J235" s="33"/>
     </row>
     <row r="236" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4528,11 +4568,11 @@
       </c>
       <c r="C236" s="10"/>
       <c r="D236" s="23"/>
-      <c r="E236" s="39"/>
+      <c r="E236" s="36"/>
       <c r="F236" s="21"/>
-      <c r="G236" s="36"/>
-      <c r="H236" s="36"/>
-      <c r="I236" s="36"/>
+      <c r="G236" s="39"/>
+      <c r="H236" s="39"/>
+      <c r="I236" s="39"/>
       <c r="J236" s="33"/>
     </row>
     <row r="237" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4543,11 +4583,11 @@
       </c>
       <c r="C237" s="10"/>
       <c r="D237" s="23"/>
-      <c r="E237" s="39"/>
+      <c r="E237" s="36"/>
       <c r="F237" s="21"/>
-      <c r="G237" s="36"/>
-      <c r="H237" s="36"/>
-      <c r="I237" s="36"/>
+      <c r="G237" s="39"/>
+      <c r="H237" s="39"/>
+      <c r="I237" s="39"/>
       <c r="J237" s="33"/>
     </row>
     <row r="238" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4558,11 +4598,11 @@
       </c>
       <c r="C238" s="10"/>
       <c r="D238" s="23"/>
-      <c r="E238" s="39"/>
+      <c r="E238" s="36"/>
       <c r="F238" s="21"/>
-      <c r="G238" s="36"/>
-      <c r="H238" s="36"/>
-      <c r="I238" s="36"/>
+      <c r="G238" s="39"/>
+      <c r="H238" s="39"/>
+      <c r="I238" s="39"/>
       <c r="J238" s="33"/>
     </row>
     <row r="239" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4573,11 +4613,11 @@
       </c>
       <c r="C239" s="10"/>
       <c r="D239" s="24"/>
-      <c r="E239" s="40"/>
+      <c r="E239" s="37"/>
       <c r="F239" s="21"/>
-      <c r="G239" s="37"/>
-      <c r="H239" s="37"/>
-      <c r="I239" s="37"/>
+      <c r="G239" s="40"/>
+      <c r="H239" s="40"/>
+      <c r="I239" s="40"/>
       <c r="J239" s="34"/>
     </row>
     <row r="240" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4590,11 +4630,11 @@
       </c>
       <c r="C240" s="10"/>
       <c r="D240" s="22"/>
-      <c r="E240" s="38"/>
+      <c r="E240" s="35"/>
       <c r="F240" s="21"/>
-      <c r="G240" s="35"/>
-      <c r="H240" s="35"/>
-      <c r="I240" s="35"/>
+      <c r="G240" s="38"/>
+      <c r="H240" s="38"/>
+      <c r="I240" s="38"/>
       <c r="J240" s="32"/>
     </row>
     <row r="241" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4605,11 +4645,11 @@
       </c>
       <c r="C241" s="10"/>
       <c r="D241" s="23"/>
-      <c r="E241" s="39"/>
+      <c r="E241" s="36"/>
       <c r="F241" s="21"/>
-      <c r="G241" s="36"/>
-      <c r="H241" s="36"/>
-      <c r="I241" s="36"/>
+      <c r="G241" s="39"/>
+      <c r="H241" s="39"/>
+      <c r="I241" s="39"/>
       <c r="J241" s="33"/>
     </row>
     <row r="242" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4620,11 +4660,11 @@
       </c>
       <c r="C242" s="10"/>
       <c r="D242" s="23"/>
-      <c r="E242" s="39"/>
+      <c r="E242" s="36"/>
       <c r="F242" s="21"/>
-      <c r="G242" s="36"/>
-      <c r="H242" s="36"/>
-      <c r="I242" s="36"/>
+      <c r="G242" s="39"/>
+      <c r="H242" s="39"/>
+      <c r="I242" s="39"/>
       <c r="J242" s="33"/>
     </row>
     <row r="243" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4635,11 +4675,11 @@
       </c>
       <c r="C243" s="10"/>
       <c r="D243" s="23"/>
-      <c r="E243" s="39"/>
+      <c r="E243" s="36"/>
       <c r="F243" s="21"/>
-      <c r="G243" s="36"/>
-      <c r="H243" s="36"/>
-      <c r="I243" s="36"/>
+      <c r="G243" s="39"/>
+      <c r="H243" s="39"/>
+      <c r="I243" s="39"/>
       <c r="J243" s="33"/>
     </row>
     <row r="244" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4650,11 +4690,11 @@
       </c>
       <c r="C244" s="10"/>
       <c r="D244" s="23"/>
-      <c r="E244" s="39"/>
+      <c r="E244" s="36"/>
       <c r="F244" s="21"/>
-      <c r="G244" s="36"/>
-      <c r="H244" s="36"/>
-      <c r="I244" s="36"/>
+      <c r="G244" s="39"/>
+      <c r="H244" s="39"/>
+      <c r="I244" s="39"/>
       <c r="J244" s="33"/>
     </row>
     <row r="245" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4665,11 +4705,11 @@
       </c>
       <c r="C245" s="10"/>
       <c r="D245" s="23"/>
-      <c r="E245" s="39"/>
+      <c r="E245" s="36"/>
       <c r="F245" s="21"/>
-      <c r="G245" s="36"/>
-      <c r="H245" s="36"/>
-      <c r="I245" s="36"/>
+      <c r="G245" s="39"/>
+      <c r="H245" s="39"/>
+      <c r="I245" s="39"/>
       <c r="J245" s="33"/>
     </row>
     <row r="246" spans="1:10" ht="10" customHeight="1" x14ac:dyDescent="0.35">
@@ -4680,11 +4720,11 @@
       </c>
       <c r="C246" s="10"/>
       <c r="D246" s="24"/>
-      <c r="E246" s="40"/>
+      <c r="E246" s="37"/>
       <c r="F246" s="21"/>
-      <c r="G246" s="37"/>
-      <c r="H246" s="37"/>
-      <c r="I246" s="37"/>
+      <c r="G246" s="40"/>
+      <c r="H246" s="40"/>
+      <c r="I246" s="40"/>
       <c r="J246" s="34"/>
     </row>
     <row r="247" spans="1:10" s="17" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
@@ -4697,7 +4737,7 @@
       </c>
       <c r="G247" s="20">
         <f t="shared" ref="G247:I247" si="4">SUM(G2:G246)</f>
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="H247" s="20">
         <f t="shared" si="4"/>
@@ -4705,7 +4745,7 @@
       </c>
       <c r="I247" s="20">
         <f t="shared" si="4"/>
-        <v>73</v>
+        <v>95</v>
       </c>
       <c r="J247" s="19"/>
     </row>
@@ -5007,12 +5047,7 @@
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="2fe66b02-ee31-4649-8513-d45fa9753ec2" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="139868d9-8e95-45bc-83ba-82132d321acb">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
+  <documentManagement/>
 </p:properties>
 </file>
 
@@ -5026,10 +5061,9 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101009D8B956648DEE047ADDF78BFAC90AFFC" ma:contentTypeVersion="18" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="ab4451092717e805e8f79af195385f10">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="139868d9-8e95-45bc-83ba-82132d321acb" xmlns:ns3="2fe66b02-ee31-4649-8513-d45fa9753ec2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0262d71ed8fd281f87c9f1c516947864" ns2:_="" ns3:_="">
-    <xsd:import namespace="139868d9-8e95-45bc-83ba-82132d321acb"/>
-    <xsd:import namespace="2fe66b02-ee31-4649-8513-d45fa9753ec2"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100ACFC688FEEC64142BC90163AE40CA300" ma:contentTypeVersion="3" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="840d1cbd9150ba30296ec1796cefda98">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3b85d9c3-74ea-4f80-8ac7-48a17b6f74b1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="617d91b5185e2c04c70a4b5d454359b0" ns2:_="">
+    <xsd:import namespace="3b85d9c3-74ea-4f80-8ac7-48a17b6f74b1"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -5038,20 +5072,7 @@
               <xsd:all>
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -5059,7 +5080,7 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="139868d9-8e95-45bc-83ba-82132d321acb" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="3b85d9c3-74ea-4f80-8ac7-48a17b6f74b1" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
@@ -5072,107 +5093,10 @@
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="14" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="16" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="18" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Bildmarkierungen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1ad04c9c-2d19-4dbf-9b4f-ffec7dfd6d5f" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="20" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceKeyPoints" ma:index="21" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="23" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="24" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2fe66b02-ee31-4649-8513-d45fa9753ec2" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="10" nillable="true" ma:displayName="Freigegeben für" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="11" nillable="true" ma:displayName="Freigegeben für - Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="TaxCatchAll" ma:index="19" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{10b003ac-eda0-4a99-9a70-2df02b00171d}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2fe66b02-ee31-4649-8513-d45fa9753ec2">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -5277,10 +5201,15 @@
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{479233DE-FAFC-4A4F-A550-35DFE1DB4063}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="2fe66b02-ee31-4649-8513-d45fa9753ec2"/>
-    <ds:schemaRef ds:uri="139868d9-8e95-45bc-83ba-82132d321acb"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="3b85d9c3-74ea-4f80-8ac7-48a17b6f74b1"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -5294,14 +5223,13 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66ED5CF9-61FE-424F-899D-F6ECF7870750}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3D6FB3BA-4B35-47AA-A75D-63FA1CA306EF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
     <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="139868d9-8e95-45bc-83ba-82132d321acb"/>
-    <ds:schemaRef ds:uri="2fe66b02-ee31-4649-8513-d45fa9753ec2"/>
+    <ds:schemaRef ds:uri="3b85d9c3-74ea-4f80-8ac7-48a17b6f74b1"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>

</xml_diff>